<commit_message>
docs: record wave zero verification evidence
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R35232bbb1dea4b98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R192b517bf09b46e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="Re17e77c5ce894e20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="R3f576eb38d3d483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R5f6c1e4ba95a4b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R6f2f0d0a80414a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R0135ac250d8f4225"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="Rd1af57dcff1a4dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="Raf4c588e6698487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra38c708042c749c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R5599d9a23e20403a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="Reb096329e9b84027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="R0c851c5b04024594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R306874276ec24b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="Rbbb27aef48464146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R562d27e3812d4b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R7623a1940b8a4f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R16c57d9f502e4d1c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -98,7 +98,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="21">
+  <x:borders count="20">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -273,16 +273,11 @@
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
     </x:border>
-    <x:border>
-      <x:bottom style="thin">
-        <x:color rgb="FFCBD5E1"/>
-      </x:bottom>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="91">
+  <x:cellXfs count="90">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -474,14 +469,13 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1058,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R963e5adf5fdf4a5f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R05a39fa0a632434f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1169,7 +1163,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Kind"/>
@@ -1781,7 +1775,7 @@
       </x:c>
       <x:c r="K23" t="n">
         <x:f>COUNTIF('Findings'!$G$2:$G$200,J23)</x:f>
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1806,7 +1800,7 @@
       </x:c>
       <x:c r="K24" t="n">
         <x:f>COUNTIF('Findings'!$G$2:$G$200,J24)</x:f>
-        <x:v>15</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1831,7 +1825,7 @@
       </x:c>
       <x:c r="K25" t="n">
         <x:f>COUNTIF('Findings'!$G$2:$G$200,J25)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1856,7 +1850,7 @@
       </x:c>
       <x:c r="K26" t="n">
         <x:f>COUNTIF('Findings'!$G$2:$G$200,J26)</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1942,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a5f63bc41d948c2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b6d446b019d400d"/>
 </x:worksheet>
 </file>
 
@@ -2026,7 +2020,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="81" t="str">
-        <x:v>observed</x:v>
+        <x:v>reproduced</x:v>
       </x:c>
       <x:c r="H2" s="81" t="str">
         <x:v>Typecheck fails; next build impossible (app/venue/equipment/page.tsx syntax error :557/:1138)</x:v>
@@ -2037,9 +2031,13 @@
       <x:c r="J2" s="81" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K2" s="81" t="str"/>
+      <x:c r="K2" s="81" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
       <x:c r="L2" s="81" t="str"/>
-      <x:c r="M2" s="81" t="str"/>
+      <x:c r="M2" s="81" t="str">
+        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="82" t="str">
@@ -2446,7 +2444,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="82" t="str">
-        <x:v>observed</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="H14" s="82" t="str">
         <x:v>Both security CI gates red: route registry 11+ unclassified (legacy ceiling 122/122); service-role allowlist 38 new bare imports</x:v>
@@ -2457,9 +2455,13 @@
       <x:c r="J14" s="82" t="str">
         <x:v>ADM-WF-017; ADM-WF-019</x:v>
       </x:c>
-      <x:c r="K14" s="82" t="str"/>
+      <x:c r="K14" s="82" t="str">
+        <x:v>Security engineering</x:v>
+      </x:c>
       <x:c r="L14" s="82" t="str"/>
-      <x:c r="M14" s="82" t="str"/>
+      <x:c r="M14" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="82" t="str">
@@ -4266,7 +4268,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G66" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H66" s="82" t="str">
         <x:v>Audit status ledger is unusable</x:v>
@@ -4277,9 +4279,13 @@
       <x:c r="J66" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K66" s="82" t="str"/>
+      <x:c r="K66" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L66" s="82" t="str"/>
-      <x:c r="M66" s="82" t="str"/>
+      <x:c r="M66" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="82" t="str">
@@ -4301,7 +4307,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G67" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H67" s="82" t="str">
         <x:v>Claimed remediation commits are unavailable</x:v>
@@ -4312,9 +4318,13 @@
       <x:c r="J67" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K67" s="82" t="str"/>
+      <x:c r="K67" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L67" s="82" t="str"/>
-      <x:c r="M67" s="82" t="str"/>
+      <x:c r="M67" s="82" t="str">
+        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="82" t="str">
@@ -4336,7 +4346,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G68" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="H68" s="82" t="str">
         <x:v>Typecheck and build evidence conflicts</x:v>
@@ -4347,9 +4357,13 @@
       <x:c r="J68" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K68" s="82" t="str"/>
+      <x:c r="K68" s="82" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
       <x:c r="L68" s="82" t="str"/>
-      <x:c r="M68" s="82" t="str"/>
+      <x:c r="M68" s="82" t="str">
+        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="82" t="str">
@@ -4371,7 +4385,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G69" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H69" s="82" t="str">
         <x:v>Finding phases and dependencies are corrupted</x:v>
@@ -4382,9 +4396,13 @@
       <x:c r="J69" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K69" s="82" t="str"/>
+      <x:c r="K69" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L69" s="82" t="str"/>
-      <x:c r="M69" s="82" t="str"/>
+      <x:c r="M69" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="82" t="str">
@@ -4406,7 +4424,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G70" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H70" s="82" t="str">
         <x:v>Mandatory phase exits were not earned</x:v>
@@ -4417,9 +4435,13 @@
       <x:c r="J70" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K70" s="82" t="str"/>
+      <x:c r="K70" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L70" s="82" t="str"/>
-      <x:c r="M70" s="82" t="str"/>
+      <x:c r="M70" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="82" t="str">
@@ -4441,7 +4463,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G71" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H71" s="82" t="str">
         <x:v>Canonical event split was mislabeled non-blocking</x:v>
@@ -4452,9 +4474,13 @@
       <x:c r="J71" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K71" s="82" t="str"/>
+      <x:c r="K71" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L71" s="82" t="str"/>
-      <x:c r="M71" s="82" t="str"/>
+      <x:c r="M71" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="82" t="str">
@@ -4511,7 +4537,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G73" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H73" s="82" t="str">
         <x:v>Three narrative findings were lost in the crosswalk</x:v>
@@ -4522,9 +4548,13 @@
       <x:c r="J73" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K73" s="82" t="str"/>
+      <x:c r="K73" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L73" s="82" t="str"/>
-      <x:c r="M73" s="82" t="str"/>
+      <x:c r="M73" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="82" t="str">
@@ -4546,7 +4576,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G74" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H74" s="82" t="str">
         <x:v>Acceptance criteria are templated rather than functional</x:v>
@@ -4557,9 +4587,13 @@
       <x:c r="J74" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K74" s="82" t="str"/>
+      <x:c r="K74" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L74" s="82" t="str"/>
-      <x:c r="M74" s="82" t="str"/>
+      <x:c r="M74" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="82" t="str">
@@ -4581,7 +4615,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G75" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H75" s="82" t="str">
         <x:v>Duplicate task and finding systems invite double counting</x:v>
@@ -4592,9 +4626,13 @@
       <x:c r="J75" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K75" s="82" t="str"/>
+      <x:c r="K75" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L75" s="82" t="str"/>
-      <x:c r="M75" s="82" t="str"/>
+      <x:c r="M75" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="82" t="str">
@@ -4616,7 +4654,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G76" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H76" s="82" t="str">
         <x:v>Source finding IDs were renamed inconsistently</x:v>
@@ -4627,9 +4665,13 @@
       <x:c r="J76" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K76" s="82" t="str"/>
+      <x:c r="K76" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L76" s="82" t="str"/>
-      <x:c r="M76" s="82" t="str"/>
+      <x:c r="M76" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="82" t="str">
@@ -4651,7 +4693,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G77" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="H77" s="82" t="str">
         <x:v>Test failure summaries are internally inconsistent</x:v>
@@ -4662,9 +4704,13 @@
       <x:c r="J77" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K77" s="82" t="str"/>
+      <x:c r="K77" s="82" t="str">
+        <x:v>Quality engineering</x:v>
+      </x:c>
       <x:c r="L77" s="82" t="str"/>
-      <x:c r="M77" s="82" t="str"/>
+      <x:c r="M77" s="82" t="str">
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="82" t="str">
@@ -4686,7 +4732,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G78" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="H78" s="82" t="str">
         <x:v>Live-audit provenance is missing</x:v>
@@ -4697,9 +4743,13 @@
       <x:c r="J78" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K78" s="82" t="str"/>
+      <x:c r="K78" s="82" t="str">
+        <x:v>Database security</x:v>
+      </x:c>
       <x:c r="L78" s="82" t="str"/>
-      <x:c r="M78" s="82" t="str"/>
+      <x:c r="M78" s="82" t="str">
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="82" t="str">
@@ -4721,7 +4771,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G79" s="82" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="H79" s="82" t="str">
         <x:v>Finding domain classifications are unreliable</x:v>
@@ -4732,9 +4782,13 @@
       <x:c r="J79" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K79" s="82" t="str"/>
+      <x:c r="K79" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L79" s="82" t="str"/>
-      <x:c r="M79" s="82" t="str"/>
+      <x:c r="M79" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="83" t="str">
@@ -4756,7 +4810,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G80" s="83" t="str">
-        <x:v>reproduced</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="H80" s="83" t="str">
         <x:v>Audit reproduction used divergent paths and dirty workspaces</x:v>
@@ -4767,9 +4821,13 @@
       <x:c r="J80" s="83" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K80" s="83" t="str"/>
+      <x:c r="K80" s="83" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="L80" s="83" t="str"/>
-      <x:c r="M80" s="83" t="str"/>
+      <x:c r="M80" s="83" t="str">
+        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C2:C80">
@@ -4794,7 +4852,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4635b0ac59647df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49afbf2c89254175"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5644,7 +5702,7 @@
         <x:v>in_scope</x:v>
       </x:c>
       <x:c r="F18" s="82" t="str">
-        <x:v>observed</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="G18" s="82" t="str">
         <x:v>PER-017</x:v>
@@ -5668,11 +5726,15 @@
         <x:v>positive; direct_data_access; idempotency; retry; rollback</x:v>
       </x:c>
       <x:c r="N18" s="82" t="str">
-        <x:v>ADM-M-001; ADM-M-013; ADM-M-018; ADM-M-019; ADM-M-038; ADM-M-048; ADM-M-049; ADM-M-058; ADM-M-061</x:v>
-      </x:c>
-      <x:c r="O18" s="82" t="str"/>
+        <x:v>ADM-M-001; ADM-M-013; ADM-M-018; ADM-M-019; ADM-M-038; ADM-M-048; ADM-M-049; ADM-M-058; ADM-M-061; AOA-001; AOA-002; AOA-003; AOA-004; AOA-005; AOA-006; AOA-007; AOA-008; AOA-009; AOA-010; AOA-011; AOA-012; AOA-013; AOA-014; AOA-015</x:v>
+      </x:c>
+      <x:c r="O18" s="82" t="str">
+        <x:v>Engineering assurance</x:v>
+      </x:c>
       <x:c r="P18" s="82" t="str"/>
-      <x:c r="Q18" s="82" t="str"/>
+      <x:c r="Q18" s="82" t="str">
+        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="82" t="str">
@@ -5827,7 +5889,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2e6f365a8ba4fcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd3b001937504e41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16776,7 +16838,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfae336081e3040f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66e1631cdc8344f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17387,7 +17449,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60b11a47b73e4a7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f28fd6fab94a3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17657,7 +17719,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb975d00635642c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d58d3a2abb74e8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17719,45 +17781,297 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="89" t="str">
+      <x:c r="A2" s="81" t="str">
         <x:v>EVD-BASELINE-CHECKPOINT</x:v>
       </x:c>
-      <x:c r="B2" s="89" t="str">
+      <x:c r="B2" s="81" t="str">
         <x:v>commit</x:v>
       </x:c>
-      <x:c r="C2" s="89" t="str">
+      <x:c r="C2" s="81" t="str">
         <x:v>pass</x:v>
       </x:c>
-      <x:c r="D2" s="89" t="str">
+      <x:c r="D2" s="81" t="str">
         <x:v>local</x:v>
       </x:c>
-      <x:c r="E2" s="90" t="n">
+      <x:c r="E2" s="87" t="n">
         <x:v>46261.39236111111</x:v>
       </x:c>
-      <x:c r="F2" s="89" t="str">
+      <x:c r="F2" s="81" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="G2" s="89" t="str">
+      <x:c r="G2" s="81" t="str">
         <x:v>a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
       </x:c>
-      <x:c r="H2" s="89" t="str">
+      <x:c r="H2" s="81" t="str">
         <x:v>git:codex/admin-workflow-completion@a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
       </x:c>
-      <x:c r="I2" s="89" t="str">
+      <x:c r="I2" s="81" t="str">
         <x:v>AOA-002; AOA-015</x:v>
       </x:c>
-      <x:c r="J2" s="89" t="str">
+      <x:c r="J2" s="81" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K2" s="89" t="str"/>
-      <x:c r="L2" s="89" t="str">
+      <x:c r="K2" s="81" t="str"/>
+      <x:c r="L2" s="81" t="str">
         <x:v>Immutable checkpoint of the 138-path August 21 workspace baseline. Human inventory sign-off remains a separate release control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="82" t="str">
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+      </x:c>
+      <x:c r="B3" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C3" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D3" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E3" s="88" t="n">
+        <x:v>46262.33998842593</x:v>
+      </x:c>
+      <x:c r="F3" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G3" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H3" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
+      </x:c>
+      <x:c r="I3" s="82" t="str">
+        <x:v>AOA-012</x:v>
+      </x:c>
+      <x:c r="J3" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K3" s="82" t="str"/>
+      <x:c r="L3" s="82" t="str">
+        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="82" t="str">
+        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+      </x:c>
+      <x:c r="B4" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C4" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D4" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E4" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F4" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G4" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H4" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
+      </x:c>
+      <x:c r="I4" s="82" t="str">
+        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+      </x:c>
+      <x:c r="J4" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K4" s="82" t="str"/>
+      <x:c r="L4" s="82" t="str">
+        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="82" t="str">
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+      </x:c>
+      <x:c r="B5" s="82" t="str">
+        <x:v>commit</x:v>
+      </x:c>
+      <x:c r="C5" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D5" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E5" s="88" t="n">
+        <x:v>46262.33961805556</x:v>
+      </x:c>
+      <x:c r="F5" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G5" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H5" s="82" t="str">
+        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="I5" s="82" t="str">
+        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
+      </x:c>
+      <x:c r="J5" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K5" s="82" t="str"/>
+      <x:c r="L5" s="82" t="str">
+        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="82" t="str">
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+      </x:c>
+      <x:c r="B6" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C6" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D6" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E6" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F6" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G6" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H6" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
+      </x:c>
+      <x:c r="I6" s="82" t="str">
+        <x:v>AOA-013; AOA-015</x:v>
+      </x:c>
+      <x:c r="J6" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K6" s="82" t="str"/>
+      <x:c r="L6" s="82" t="str">
+        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="82" t="str">
+        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+      </x:c>
+      <x:c r="B7" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C7" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D7" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E7" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F7" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G7" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H7" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+      </x:c>
+      <x:c r="I7" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J7" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K7" s="82" t="str"/>
+      <x:c r="L7" s="82" t="str">
+        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="82" t="str">
+        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+      </x:c>
+      <x:c r="B8" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C8" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D8" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E8" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F8" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G8" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H8" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+      </x:c>
+      <x:c r="I8" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J8" s="82" t="str">
+        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="K8" s="82" t="str"/>
+      <x:c r="L8" s="82" t="str">
+        <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="83" t="str">
+        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+      </x:c>
+      <x:c r="B9" s="83" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C9" s="83" t="str">
+        <x:v>fail</x:v>
+      </x:c>
+      <x:c r="D9" s="83" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E9" s="89" t="n">
+        <x:v>46262.33513888889</x:v>
+      </x:c>
+      <x:c r="F9" s="83" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G9" s="83" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H9" s="83" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
+      </x:c>
+      <x:c r="I9" s="83" t="str">
+        <x:v>ADM-M-001; AOA-003</x:v>
+      </x:c>
+      <x:c r="J9" s="83" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K9" s="83" t="str"/>
+      <x:c r="L9" s="83" t="str">
+        <x:v>Pinned Node 20 full-repository typecheck exited 2 after 2,652.36 seconds. It checked 7,456 files, used about 6.3 GB, and reported type/schema drift across Admin and non-Admin code; the captured command output contained 3,005 lines. LG-01 remains not verified and the production build was not attempted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14360f92e8144497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb47aba062974cf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18000,7 +18314,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30687d84c7924822"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cd51bb56dea4cf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18573,7 +18887,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cb78760a5df4640"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra438e4ed6e764e06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: enforce admin site map read capabilities
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra38c708042c749c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R5599d9a23e20403a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="Reb096329e9b84027"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="R0c851c5b04024594"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R306874276ec24b6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="Rbbb27aef48464146"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R562d27e3812d4b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R7623a1940b8a4f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R16c57d9f502e4d1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdb7602a4605e4a11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R2c37b2bba4f0477e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R40db7318d341493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="R9105cfdc16024bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="Rd19c528ee1694e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R483a9a6029164b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R5b9bc271afb841d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R8db71240c8b34f87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R4baf1ace78d646e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1052,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R05a39fa0a632434f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2a272ccad8c846c5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1936,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b6d446b019d400d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c11de4df074c0d"/>
 </x:worksheet>
 </file>
 
@@ -4852,7 +4852,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49afbf2c89254175"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e586e647fb4ba4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5889,7 +5889,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd3b001937504e41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4650a7fd23d24f9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16838,7 +16838,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66e1631cdc8344f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra99a27ba144541ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17449,7 +17449,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f28fd6fab94a3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d82e22df9074e78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17719,7 +17719,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d58d3a2abb74e8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaff066734ce4dec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18071,7 +18071,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb47aba062974cf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bf1d31138544e94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18314,7 +18314,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cd51bb56dea4cf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R485f0f04a9ac4426"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18887,7 +18887,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra438e4ed6e764e06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfce486b9feab411e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record site map capability evidence
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdb7602a4605e4a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R2c37b2bba4f0477e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R40db7318d341493f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="R9105cfdc16024bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="Rd19c528ee1694e68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R483a9a6029164b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R5b9bc271afb841d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R8db71240c8b34f87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R4baf1ace78d646e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R89d5ce5048904261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R7c4c6830ec8e45f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R8cf42d117d794b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rd264f80f370d40af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R896c1c22d04a404f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R00c7c0669b3e4f5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R8aeb589fc7fd4151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R2aa8a44d04cd4f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R0b3d4f9af24949ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1052,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2a272ccad8c846c5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1af9e7ce1da4a8a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1163,7 +1163,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Kind"/>
@@ -1936,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c11de4df074c0d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ffe93588f5c43dd"/>
 </x:worksheet>
 </file>
 
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="L14" s="82" t="str"/>
       <x:c r="M14" s="82" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4852,7 +4852,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e586e647fb4ba4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7e602fe75634752"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5514,7 +5514,7 @@
         <x:v>in_scope</x:v>
       </x:c>
       <x:c r="F14" s="82" t="str">
-        <x:v>observed</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="G14" s="82" t="str">
         <x:v>PER-002</x:v>
@@ -5538,11 +5538,15 @@
         <x:v>positive; recipient; cross_org; tamper; revoked; unauthenticated; direct_data_access; idempotency; retry; rollback</x:v>
       </x:c>
       <x:c r="N14" s="82" t="str">
-        <x:v>ADM-M-002; ADM-M-010; ADM-M-011; ADM-M-038; ADM-M-061</x:v>
-      </x:c>
-      <x:c r="O14" s="82" t="str"/>
+        <x:v>ADM-M-002; ADM-M-010; ADM-M-011; ADM-M-013; ADM-M-038; ADM-M-061</x:v>
+      </x:c>
+      <x:c r="O14" s="82" t="str">
+        <x:v>Operations engineering</x:v>
+      </x:c>
       <x:c r="P14" s="82" t="str"/>
-      <x:c r="Q14" s="82" t="str"/>
+      <x:c r="Q14" s="82" t="str">
+        <x:v>EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="82" t="str">
@@ -5733,7 +5737,7 @@
       </x:c>
       <x:c r="P18" s="82" t="str"/>
       <x:c r="Q18" s="82" t="str">
-        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5889,7 +5893,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4650a7fd23d24f9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d54494cdb5b4049"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16838,7 +16842,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra99a27ba144541ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfa8b7b7189f4752"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17449,7 +17453,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d82e22df9074e78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2486fd21ca4dac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17719,7 +17723,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaff066734ce4dec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09196a885d0c42af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17818,10 +17822,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="82" t="str">
-        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
       </x:c>
       <x:c r="B3" s="82" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C3" s="82" t="str">
         <x:v>pass</x:v>
@@ -17830,31 +17834,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E3" s="88" t="n">
-        <x:v>46262.33998842593</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F3" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G3" s="82" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H3" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
+        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="I3" s="82" t="str">
-        <x:v>AOA-012</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J3" s="82" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K3" s="82" t="str"/>
       <x:c r="L3" s="82" t="str">
-        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="82" t="str">
-        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
       <x:c r="B4" s="82" t="str">
         <x:v>test_run</x:v>
@@ -17866,34 +17870,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E4" s="88" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F4" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G4" s="82" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H4" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
+        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I4" s="82" t="str">
-        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J4" s="82" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K4" s="82" t="str"/>
       <x:c r="L4" s="82" t="str">
-        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
+        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="82" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
       </x:c>
       <x:c r="B5" s="82" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C5" s="82" t="str">
         <x:v>pass</x:v>
@@ -17902,7 +17906,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E5" s="88" t="n">
-        <x:v>46262.33961805556</x:v>
+        <x:v>46262.33998842593</x:v>
       </x:c>
       <x:c r="F5" s="82" t="str">
         <x:v>Codex</x:v>
@@ -17911,22 +17915,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H5" s="82" t="str">
-        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
       </x:c>
       <x:c r="I5" s="82" t="str">
-        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
+        <x:v>AOA-012</x:v>
       </x:c>
       <x:c r="J5" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K5" s="82" t="str"/>
       <x:c r="L5" s="82" t="str">
-        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
+        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="82" t="str">
-        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B6" s="82" t="str">
         <x:v>test_run</x:v>
@@ -17947,25 +17951,25 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H6" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
       </x:c>
       <x:c r="I6" s="82" t="str">
-        <x:v>AOA-013; AOA-015</x:v>
+        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J6" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K6" s="82" t="str"/>
       <x:c r="L6" s="82" t="str">
-        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="82" t="str">
-        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
       </x:c>
       <x:c r="B7" s="82" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C7" s="82" t="str">
         <x:v>pass</x:v>
@@ -17974,7 +17978,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E7" s="88" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.33961805556</x:v>
       </x:c>
       <x:c r="F7" s="82" t="str">
         <x:v>Codex</x:v>
@@ -17983,22 +17987,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H7" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="I7" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
       </x:c>
       <x:c r="J7" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K7" s="82" t="str"/>
       <x:c r="L7" s="82" t="str">
-        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="82" t="str">
-        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
       </x:c>
       <x:c r="B8" s="82" t="str">
         <x:v>test_run</x:v>
@@ -18019,59 +18023,131 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H8" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
       </x:c>
       <x:c r="I8" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>AOA-013; AOA-015</x:v>
       </x:c>
       <x:c r="J8" s="82" t="str">
-        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K8" s="82" t="str"/>
       <x:c r="L8" s="82" t="str">
+        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="82" t="str">
+        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+      </x:c>
+      <x:c r="B9" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C9" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D9" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E9" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F9" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G9" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H9" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+      </x:c>
+      <x:c r="I9" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J9" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K9" s="82" t="str"/>
+      <x:c r="L9" s="82" t="str">
+        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="82" t="str">
+        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+      </x:c>
+      <x:c r="B10" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C10" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D10" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E10" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F10" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G10" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H10" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+      </x:c>
+      <x:c r="I10" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J10" s="82" t="str">
+        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="K10" s="82" t="str"/>
+      <x:c r="L10" s="82" t="str">
         <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="83" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="83" t="str">
         <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
       </x:c>
-      <x:c r="B9" s="83" t="str">
+      <x:c r="B11" s="83" t="str">
         <x:v>test_run</x:v>
       </x:c>
-      <x:c r="C9" s="83" t="str">
+      <x:c r="C11" s="83" t="str">
         <x:v>fail</x:v>
       </x:c>
-      <x:c r="D9" s="83" t="str">
+      <x:c r="D11" s="83" t="str">
         <x:v>local</x:v>
       </x:c>
-      <x:c r="E9" s="89" t="n">
+      <x:c r="E11" s="89" t="n">
         <x:v>46262.33513888889</x:v>
       </x:c>
-      <x:c r="F9" s="83" t="str">
+      <x:c r="F11" s="83" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="G9" s="83" t="str">
+      <x:c r="G11" s="83" t="str">
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
-      <x:c r="H9" s="83" t="str">
+      <x:c r="H11" s="83" t="str">
         <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
       </x:c>
-      <x:c r="I9" s="83" t="str">
+      <x:c r="I11" s="83" t="str">
         <x:v>ADM-M-001; AOA-003</x:v>
       </x:c>
-      <x:c r="J9" s="83" t="str">
+      <x:c r="J11" s="83" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K9" s="83" t="str"/>
-      <x:c r="L9" s="83" t="str">
+      <x:c r="K11" s="83" t="str"/>
+      <x:c r="L11" s="83" t="str">
         <x:v>Pinned Node 20 full-repository typecheck exited 2 after 2,652.36 seconds. It checked 7,456 files, used about 6.3 GB, and reported type/schema drift across Admin and non-Admin code; the captured command output contained 3,005 lines. LG-01 remains not verified and the production build was not attempted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bf1d31138544e94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f416c9151044d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18314,7 +18390,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R485f0f04a9ac4426"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12d1950a565e4857"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18887,7 +18963,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfce486b9feab411e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e721bd23de347d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: bind admin site maps to acting organization
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R89d5ce5048904261"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R7c4c6830ec8e45f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R8cf42d117d794b88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rd264f80f370d40af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R896c1c22d04a404f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R00c7c0669b3e4f5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R8aeb589fc7fd4151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R2aa8a44d04cd4f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R0b3d4f9af24949ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb0e7d49619254cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R07a4846ff6114370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="Rc8c7fba10cc74719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rf747d8b05b7a4294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="Rc8f5d24e9e6c45f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R3b35f3e888f8481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R8f89e91b581344cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R6c583780e7ce47ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R5d5c5b0069e64086"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1052,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1af9e7ce1da4a8a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcaef3d2dd4634d40"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1936,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ffe93588f5c43dd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2fb7854d63f4b57"/>
 </x:worksheet>
 </file>
 
@@ -4852,7 +4852,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7e602fe75634752"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb122f0bbd6d343a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5893,7 +5893,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d54494cdb5b4049"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df986c2480e4a5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16842,7 +16842,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfa8b7b7189f4752"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R056448fd7dea44c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17453,7 +17453,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2486fd21ca4dac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4303af0ac554e22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17723,7 +17723,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09196a885d0c42af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46575a468514a8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18147,7 +18147,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f416c9151044d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08880d3f07bc42bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18390,7 +18390,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12d1950a565e4857"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfa6c2d24d14a57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18963,7 +18963,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e721bd23de347d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02d3442cfbd547c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record site map organization binding evidence
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb0e7d49619254cdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R07a4846ff6114370"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="Rc8c7fba10cc74719"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rf747d8b05b7a4294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="Rc8f5d24e9e6c45f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R3b35f3e888f8481c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R8f89e91b581344cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R6c583780e7ce47ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R5d5c5b0069e64086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R09e2a57fcd4f4f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R495a11eb05ec4246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R8a9bef3447d8467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rd1069d0524af4071"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R8a93c16c623c4b25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="Rd524b81093cf4a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="Ra9450f38a46941f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R629f16b4b26c4588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="Rafdcb86b29fe4193"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1052,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcaef3d2dd4634d40"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re2e8ee8506cc496f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1163,7 +1163,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Kind"/>
@@ -1775,7 +1775,7 @@
       </x:c>
       <x:c r="K23" t="n">
         <x:f>COUNTIF('Findings'!$G$2:$G$200,J23)</x:f>
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1825,7 +1825,7 @@
       </x:c>
       <x:c r="K25" t="n">
         <x:f>COUNTIF('Findings'!$G$2:$G$200,J25)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1936,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2fb7854d63f4b57"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eece237558b4e96"/>
 </x:worksheet>
 </file>
 
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="L14" s="82" t="str"/>
       <x:c r="M14" s="82" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2658,7 +2658,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G20" s="82" t="str">
-        <x:v>observed</x:v>
+        <x:v>in_progress</x:v>
       </x:c>
       <x:c r="H20" s="82" t="str">
         <x:v>Audit logging: ~6/288 admin route files write audit rows despite central helpers</x:v>
@@ -2669,9 +2669,13 @@
       <x:c r="J20" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K20" s="82" t="str"/>
+      <x:c r="K20" s="82" t="str">
+        <x:v>Security engineering</x:v>
+      </x:c>
       <x:c r="L20" s="82" t="str"/>
-      <x:c r="M20" s="82" t="str"/>
+      <x:c r="M20" s="82" t="str">
+        <x:v>EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="82" t="str">
@@ -4852,7 +4856,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb122f0bbd6d343a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R286bf72a37614b9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5545,7 +5549,7 @@
       </x:c>
       <x:c r="P14" s="82" t="str"/>
       <x:c r="Q14" s="82" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -5737,7 +5741,7 @@
       </x:c>
       <x:c r="P18" s="82" t="str"/>
       <x:c r="Q18" s="82" t="str">
-        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5893,7 +5897,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df986c2480e4a5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d405349cf7a420c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16842,7 +16846,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R056448fd7dea44c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58fbedb09bb24540"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17453,7 +17457,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4303af0ac554e22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2188d697d43a420f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17723,7 +17727,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46575a468514a8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c804d6af27f49cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17822,7 +17826,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="82" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ACTING-COMMIT</x:v>
       </x:c>
       <x:c r="B3" s="82" t="str">
         <x:v>commit</x:v>
@@ -17834,31 +17838,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E3" s="88" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46262.35711805556</x:v>
       </x:c>
       <x:c r="F3" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G3" s="82" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="H3" s="82" t="str">
-        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>git:codex/admin-workflow-completion@abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="I3" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J3" s="82" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K3" s="82" t="str"/>
       <x:c r="L3" s="82" t="str">
-        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
+        <x:v>Immutable SEC-104 checkpoint binding linked site maps to the acting organization and replacing the generic activity writer with validated, actor-bound commands.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="82" t="str">
-        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
       </x:c>
       <x:c r="B4" s="82" t="str">
         <x:v>test_run</x:v>
@@ -17870,34 +17874,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E4" s="88" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46262.35711805556</x:v>
       </x:c>
       <x:c r="F4" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G4" s="82" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="H4" s="82" t="str">
-        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
+        <x:v>Node 20 route registry, focused active-org/tamper/actor-binding tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I4" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J4" s="82" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K4" s="82" t="str"/>
       <x:c r="L4" s="82" t="str">
-        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
+        <x:v>Local verification passed: 288 routes at 113/113 legacy; linked Org A/Org B mismatch and unscoped-map denial; forged activity action/actor/status rejection; child-map ownership; 230 active Admin files and 3,218 active tests. Live RLS and staging remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="82" t="str">
-        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
       </x:c>
       <x:c r="B5" s="82" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C5" s="82" t="str">
         <x:v>pass</x:v>
@@ -17906,31 +17910,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E5" s="88" t="n">
-        <x:v>46262.33998842593</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F5" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G5" s="82" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H5" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
+        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="I5" s="82" t="str">
-        <x:v>AOA-012</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J5" s="82" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K5" s="82" t="str"/>
       <x:c r="L5" s="82" t="str">
-        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="82" t="str">
-        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
       <x:c r="B6" s="82" t="str">
         <x:v>test_run</x:v>
@@ -17942,34 +17946,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E6" s="88" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F6" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G6" s="82" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H6" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
+        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I6" s="82" t="str">
-        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J6" s="82" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K6" s="82" t="str"/>
       <x:c r="L6" s="82" t="str">
-        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
+        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="82" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
       </x:c>
       <x:c r="B7" s="82" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C7" s="82" t="str">
         <x:v>pass</x:v>
@@ -17978,7 +17982,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E7" s="88" t="n">
-        <x:v>46262.33961805556</x:v>
+        <x:v>46262.33998842593</x:v>
       </x:c>
       <x:c r="F7" s="82" t="str">
         <x:v>Codex</x:v>
@@ -17987,22 +17991,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H7" s="82" t="str">
-        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
       </x:c>
       <x:c r="I7" s="82" t="str">
-        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
+        <x:v>AOA-012</x:v>
       </x:c>
       <x:c r="J7" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K7" s="82" t="str"/>
       <x:c r="L7" s="82" t="str">
-        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
+        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="82" t="str">
-        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B8" s="82" t="str">
         <x:v>test_run</x:v>
@@ -18023,25 +18027,25 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H8" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
       </x:c>
       <x:c r="I8" s="82" t="str">
-        <x:v>AOA-013; AOA-015</x:v>
+        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J8" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K8" s="82" t="str"/>
       <x:c r="L8" s="82" t="str">
-        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="82" t="str">
-        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
       </x:c>
       <x:c r="B9" s="82" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C9" s="82" t="str">
         <x:v>pass</x:v>
@@ -18050,7 +18054,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E9" s="88" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.33961805556</x:v>
       </x:c>
       <x:c r="F9" s="82" t="str">
         <x:v>Codex</x:v>
@@ -18059,22 +18063,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H9" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="I9" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
       </x:c>
       <x:c r="J9" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K9" s="82" t="str"/>
       <x:c r="L9" s="82" t="str">
-        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="82" t="str">
-        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
       </x:c>
       <x:c r="B10" s="82" t="str">
         <x:v>test_run</x:v>
@@ -18095,59 +18099,131 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H10" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
       </x:c>
       <x:c r="I10" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>AOA-013; AOA-015</x:v>
       </x:c>
       <x:c r="J10" s="82" t="str">
-        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K10" s="82" t="str"/>
       <x:c r="L10" s="82" t="str">
+        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="82" t="str">
+        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+      </x:c>
+      <x:c r="B11" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C11" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D11" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E11" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F11" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G11" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H11" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+      </x:c>
+      <x:c r="I11" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J11" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K11" s="82" t="str"/>
+      <x:c r="L11" s="82" t="str">
+        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="82" t="str">
+        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+      </x:c>
+      <x:c r="B12" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C12" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D12" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E12" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F12" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G12" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H12" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+      </x:c>
+      <x:c r="I12" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J12" s="82" t="str">
+        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="K12" s="82" t="str"/>
+      <x:c r="L12" s="82" t="str">
         <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="83" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="83" t="str">
         <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
       </x:c>
-      <x:c r="B11" s="83" t="str">
+      <x:c r="B13" s="83" t="str">
         <x:v>test_run</x:v>
       </x:c>
-      <x:c r="C11" s="83" t="str">
+      <x:c r="C13" s="83" t="str">
         <x:v>fail</x:v>
       </x:c>
-      <x:c r="D11" s="83" t="str">
+      <x:c r="D13" s="83" t="str">
         <x:v>local</x:v>
       </x:c>
-      <x:c r="E11" s="89" t="n">
+      <x:c r="E13" s="89" t="n">
         <x:v>46262.33513888889</x:v>
       </x:c>
-      <x:c r="F11" s="83" t="str">
+      <x:c r="F13" s="83" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="G11" s="83" t="str">
+      <x:c r="G13" s="83" t="str">
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
-      <x:c r="H11" s="83" t="str">
+      <x:c r="H13" s="83" t="str">
         <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
       </x:c>
-      <x:c r="I11" s="83" t="str">
+      <x:c r="I13" s="83" t="str">
         <x:v>ADM-M-001; AOA-003</x:v>
       </x:c>
-      <x:c r="J11" s="83" t="str">
+      <x:c r="J13" s="83" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K11" s="83" t="str"/>
-      <x:c r="L11" s="83" t="str">
+      <x:c r="K13" s="83" t="str"/>
+      <x:c r="L13" s="83" t="str">
         <x:v>Pinned Node 20 full-repository typecheck exited 2 after 2,652.36 seconds. It checked 7,456 files, used about 6.3 GB, and reported type/schema drift across Admin and non-Admin code; the captured command output contained 3,005 lines. LG-01 remains not verified and the production build was not attempted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08880d3f07bc42bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a46bb40f65b448c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18390,7 +18466,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfa6c2d24d14a57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8fb3e752f4648b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18963,7 +19039,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02d3442cfbd547c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc60eda9e1754676"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: scope admin site map collaborators
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R09e2a57fcd4f4f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R495a11eb05ec4246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R8a9bef3447d8467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rd1069d0524af4071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R8a93c16c623c4b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="Rd524b81093cf4a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="Ra9450f38a46941f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R629f16b4b26c4588"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="Rafdcb86b29fe4193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd921af28863b4de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R0d90814983ca4119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R0ed8d533dab44653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rfe80683dc66a43d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R3e2738ebb7d941f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R726a03cbb9254be1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R740e2196e24648bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R59ab56339c1e4bf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="Rd2dcbd769fa94d43"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1052,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re2e8ee8506cc496f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra107f554ae954680"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1936,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eece237558b4e96"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94191690f0fa4434"/>
 </x:worksheet>
 </file>
 
@@ -4856,7 +4856,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R286bf72a37614b9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd248791f766940ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5897,7 +5897,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d405349cf7a420c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re14d7ff91f224224"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16846,7 +16846,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58fbedb09bb24540"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea0b7af77efb4ffe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17457,7 +17457,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2188d697d43a420f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39dce0f247bf4603"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17727,7 +17727,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c804d6af27f49cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06c8ca710307469e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18223,7 +18223,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a46bb40f65b448c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ec344e55f5422a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18466,7 +18466,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8fb3e752f4648b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b39dab4e514e42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19039,7 +19039,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc60eda9e1754676"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59746ac377eb4988"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record site map collaborator evidence
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd921af28863b4de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R0d90814983ca4119"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R0ed8d533dab44653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Rfe80683dc66a43d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R3e2738ebb7d941f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R726a03cbb9254be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R740e2196e24648bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R59ab56339c1e4bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="Rd2dcbd769fa94d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R02a58ebf913f4f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R1e05762c4d0646b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R62ea01cf37c14a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="R26522985434744cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="Re9547be8bda84b26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="Rc668bff2df7c4e8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R57a4cafa881042f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R8209082295c94499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="Ra91677ea407b4b60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1052,7 +1052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra107f554ae954680"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R05c8c1833c02405d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1163,7 +1163,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AdminEvidenceTable" displayName="AdminEvidenceTable" ref="A1:L15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Kind"/>
@@ -1936,7 +1936,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94191690f0fa4434"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a6899478d624739"/>
 </x:worksheet>
 </file>
 
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="L14" s="82" t="str"/>
       <x:c r="M14" s="82" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL; EVD-SEC104-SITEMAP-COLLAB-COMMIT; EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4856,7 +4856,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd248791f766940ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd27bf5bc76ea4a22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5549,7 +5549,7 @@
       </x:c>
       <x:c r="P14" s="82" t="str"/>
       <x:c r="Q14" s="82" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL; EVD-SEC104-SITEMAP-COLLAB-COMMIT; EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -5741,7 +5741,7 @@
       </x:c>
       <x:c r="P18" s="82" t="str"/>
       <x:c r="Q18" s="82" t="str">
-        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
+        <x:v>EVD-BASELINE-CHECKPOINT; EVD-WAVE0-CONTROLS-COMMIT; EVD-WAVE0-AUDIT-REGISTRY-LOCAL; EVD-WAVE0-ADMIN-TESTS-LOCAL; EVD-WAVE0-ROUTE-REGISTRY-LOCAL; EVD-WAVE0-SERVICE-ROLE-LOCAL; EVD-WAVE0-MIGRATIONS-LOCAL; EVD-WAVE0-TYPECHECK-LOCAL-FAIL; EVD-SEC104-SITEMAP-COMMIT; EVD-SEC104-SITEMAP-LOCAL; EVD-SEC104-SITEMAP-ACTING-COMMIT; EVD-SEC104-SITEMAP-ACTING-LOCAL; EVD-SEC104-SITEMAP-COLLAB-COMMIT; EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5897,7 +5897,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re14d7ff91f224224"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61d9acc3acc44db9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16846,7 +16846,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea0b7af77efb4ffe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dbb030c44224941"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17457,7 +17457,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39dce0f247bf4603"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb996830efa4049c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17727,7 +17727,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06c8ca710307469e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4534d60b4ec4091"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17898,7 +17898,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="82" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COLLAB-COMMIT</x:v>
       </x:c>
       <x:c r="B5" s="82" t="str">
         <x:v>commit</x:v>
@@ -17910,16 +17910,16 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E5" s="88" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46262.3608912037</x:v>
       </x:c>
       <x:c r="F5" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G5" s="82" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="H5" s="82" t="str">
-        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>git:codex/admin-workflow-completion@63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="I5" s="82" t="str">
         <x:v>ADM-M-013</x:v>
@@ -17929,12 +17929,12 @@
       </x:c>
       <x:c r="K5" s="82" t="str"/>
       <x:c r="L5" s="82" t="str">
-        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map collaborator reads/removals to active-org capabilities while preserving owner-only removal.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="82" t="str">
-        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
       </x:c>
       <x:c r="B6" s="82" t="str">
         <x:v>test_run</x:v>
@@ -17946,16 +17946,16 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E6" s="88" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46262.3608912037</x:v>
       </x:c>
       <x:c r="F6" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G6" s="82" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="H6" s="82" t="str">
-        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
+        <x:v>Node 20 route registry, collaborator input/source tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I6" s="82" t="str">
         <x:v>ADM-M-013</x:v>
@@ -17965,15 +17965,15 @@
       </x:c>
       <x:c r="K6" s="82" t="str"/>
       <x:c r="L6" s="82" t="str">
-        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
+        <x:v>Local verification passed: 288 routes at 112/112 legacy; strict collaborator UUID/tamper rejection; active-org plus owner-only removal boundary; 231 active Admin files and 3,223 active tests. Live RLS and staging remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="82" t="str">
-        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
       </x:c>
       <x:c r="B7" s="82" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C7" s="82" t="str">
         <x:v>pass</x:v>
@@ -17982,31 +17982,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E7" s="88" t="n">
-        <x:v>46262.33998842593</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F7" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G7" s="82" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H7" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
+        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="I7" s="82" t="str">
-        <x:v>AOA-012</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J7" s="82" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K7" s="82" t="str"/>
       <x:c r="L7" s="82" t="str">
-        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="82" t="str">
-        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
       <x:c r="B8" s="82" t="str">
         <x:v>test_run</x:v>
@@ -18018,34 +18018,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E8" s="88" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F8" s="82" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G8" s="82" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H8" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
+        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I8" s="82" t="str">
-        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J8" s="82" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K8" s="82" t="str"/>
       <x:c r="L8" s="82" t="str">
-        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
+        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="82" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
       </x:c>
       <x:c r="B9" s="82" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C9" s="82" t="str">
         <x:v>pass</x:v>
@@ -18054,7 +18054,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E9" s="88" t="n">
-        <x:v>46262.33961805556</x:v>
+        <x:v>46262.33998842593</x:v>
       </x:c>
       <x:c r="F9" s="82" t="str">
         <x:v>Codex</x:v>
@@ -18063,22 +18063,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H9" s="82" t="str">
-        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
       </x:c>
       <x:c r="I9" s="82" t="str">
-        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
+        <x:v>AOA-012</x:v>
       </x:c>
       <x:c r="J9" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K9" s="82" t="str"/>
       <x:c r="L9" s="82" t="str">
-        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
+        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="82" t="str">
-        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B10" s="82" t="str">
         <x:v>test_run</x:v>
@@ -18099,25 +18099,25 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H10" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
       </x:c>
       <x:c r="I10" s="82" t="str">
-        <x:v>AOA-013; AOA-015</x:v>
+        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J10" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K10" s="82" t="str"/>
       <x:c r="L10" s="82" t="str">
-        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="82" t="str">
-        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
       </x:c>
       <x:c r="B11" s="82" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C11" s="82" t="str">
         <x:v>pass</x:v>
@@ -18126,7 +18126,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E11" s="88" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.33961805556</x:v>
       </x:c>
       <x:c r="F11" s="82" t="str">
         <x:v>Codex</x:v>
@@ -18135,22 +18135,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H11" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="I11" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
       </x:c>
       <x:c r="J11" s="82" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K11" s="82" t="str"/>
       <x:c r="L11" s="82" t="str">
-        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="82" t="str">
-        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
       </x:c>
       <x:c r="B12" s="82" t="str">
         <x:v>test_run</x:v>
@@ -18171,59 +18171,131 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H12" s="82" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
       </x:c>
       <x:c r="I12" s="82" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>AOA-013; AOA-015</x:v>
       </x:c>
       <x:c r="J12" s="82" t="str">
-        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K12" s="82" t="str"/>
       <x:c r="L12" s="82" t="str">
+        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="82" t="str">
+        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+      </x:c>
+      <x:c r="B13" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C13" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D13" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E13" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F13" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G13" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H13" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+      </x:c>
+      <x:c r="I13" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J13" s="82" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K13" s="82" t="str"/>
+      <x:c r="L13" s="82" t="str">
+        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="82" t="str">
+        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+      </x:c>
+      <x:c r="B14" s="82" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C14" s="82" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D14" s="82" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E14" s="88" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F14" s="82" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G14" s="82" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H14" s="82" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+      </x:c>
+      <x:c r="I14" s="82" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J14" s="82" t="str">
+        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="K14" s="82" t="str"/>
+      <x:c r="L14" s="82" t="str">
         <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="83" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="83" t="str">
         <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
       </x:c>
-      <x:c r="B13" s="83" t="str">
+      <x:c r="B15" s="83" t="str">
         <x:v>test_run</x:v>
       </x:c>
-      <x:c r="C13" s="83" t="str">
+      <x:c r="C15" s="83" t="str">
         <x:v>fail</x:v>
       </x:c>
-      <x:c r="D13" s="83" t="str">
+      <x:c r="D15" s="83" t="str">
         <x:v>local</x:v>
       </x:c>
-      <x:c r="E13" s="89" t="n">
+      <x:c r="E15" s="89" t="n">
         <x:v>46262.33513888889</x:v>
       </x:c>
-      <x:c r="F13" s="83" t="str">
+      <x:c r="F15" s="83" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="G13" s="83" t="str">
+      <x:c r="G15" s="83" t="str">
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
-      <x:c r="H13" s="83" t="str">
+      <x:c r="H15" s="83" t="str">
         <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
       </x:c>
-      <x:c r="I13" s="83" t="str">
+      <x:c r="I15" s="83" t="str">
         <x:v>ADM-M-001; AOA-003</x:v>
       </x:c>
-      <x:c r="J13" s="83" t="str">
+      <x:c r="J15" s="83" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
-      <x:c r="K13" s="83" t="str"/>
-      <x:c r="L13" s="83" t="str">
+      <x:c r="K15" s="83" t="str"/>
+      <x:c r="L15" s="83" t="str">
         <x:v>Pinned Node 20 full-repository typecheck exited 2 after 2,652.36 seconds. It checked 7,456 files, used about 6.3 GB, and reported type/schema drift across Admin and non-Admin code; the captured command output contained 3,005 lines. LG-01 remains not verified and the production build was not attempted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ec344e55f5422a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R513a256b4355498a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18466,7 +18538,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b39dab4e514e42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7489dd9989149ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19039,7 +19111,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59746ac377eb4988"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fd53329b6d4823"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(admin): add token-efficient execution control plane
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R82b2d5e0ff124314"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="Rfd0f8515afd14d11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="3" r:id="R8f65a8ab37d6477a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="4" r:id="Raad4d521bf204703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="5" r:id="R5e7a0f86f82e4c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R32ac8fcb8bf742da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R31f802dd67934c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="Re1a21db8b00d4290"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="9" r:id="R4eac40c07f234e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbb089974eab643ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="Rb20779da8c53452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="R800f2532a5934f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R9c83015765fb4bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R4ee3b864f5524a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="Rb4eeb0e239274aa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R7c90c056dcbd494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="Rb4aa602a9acc4d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R3d53a2fe7c56450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="Rf7722bebe23042a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -839,7 +840,106 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="86">
+  <x:dxfs count="95">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF15803D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF15803D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1D4ED8"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF6D28D9"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEDE9FE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB45309"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC2410C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFEDD5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF334155"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF1F5F9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF15803D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1791,7 +1891,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DashboardGateSummary" displayName="DashboardGateSummary" ref="A13:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="DashboardGateSummary" displayName="DashboardGateSummary" ref="A13:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Gate ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1803,7 +1903,26 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AuditRisks" displayName="AuditRisks" ref="A1:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AuditLaunchGates" displayName="AuditLaunchGates" ref="A1:J19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J19"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="Gate ID"/>
+    <x:tableColumn id="2" name="Title"/>
+    <x:tableColumn id="3" name="Wave"/>
+    <x:tableColumn id="4" name="Check kind"/>
+    <x:tableColumn id="5" name="Command"/>
+    <x:tableColumn id="6" name="Acceptance"/>
+    <x:tableColumn id="7" name="Evidence kinds"/>
+    <x:tableColumn id="8" name="Dependencies"/>
+    <x:tableColumn id="9" name="Owner"/>
+    <x:tableColumn id="10" name="Evidence status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AuditRisks" displayName="AuditRisks" ref="A1:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:K7"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Risk ID"/>
@@ -1822,8 +1941,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AuditEvidence" displayName="AuditEvidence" ref="A1:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditEvidence" displayName="AuditEvidence" ref="A1:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:L19"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
@@ -1843,8 +1962,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditDecisions" displayName="AuditDecisions" ref="A1:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="AuditDecisions" displayName="AuditDecisions" ref="A1:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G10"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Decision ID"/>
@@ -1859,8 +1978,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="AuditServiceRoleDebt" displayName="AuditServiceRoleDebt" ref="A1:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AuditServiceRoleDebt" displayName="AuditServiceRoleDebt" ref="A1:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G24"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="File"/>
@@ -1876,7 +1995,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="DashboardFindingStatus" displayName="DashboardFindingStatus" ref="F13:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DashboardFindingStatus" displayName="DashboardFindingStatus" ref="F13:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Count"/>
@@ -1886,7 +2005,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DashboardWorkflowStatus" displayName="DashboardWorkflowStatus" ref="F23:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="DashboardWorkflowStatus" displayName="DashboardWorkflowStatus" ref="F23:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Count"/>
@@ -1896,7 +2015,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="DashboardPriorityMix" displayName="DashboardPriorityMix" ref="I13:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="DashboardPriorityMix" displayName="DashboardPriorityMix" ref="I13:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Priority"/>
     <x:tableColumn id="2" name="Count"/>
@@ -1906,7 +2025,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="DashboardServiceRoleDisposition" displayName="DashboardServiceRoleDisposition" ref="I20:J24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DashboardServiceRoleDisposition" displayName="DashboardServiceRoleDisposition" ref="I20:J24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Disposition"/>
     <x:tableColumn id="2" name="Count"/>
@@ -1916,7 +2035,28 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AuditFindings" displayName="AuditFindings" ref="A1:M80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AdminExecutionBatches" displayName="AdminExecutionBatches" ref="A1:L16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L16"/>
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Batch ID"/>
+    <x:tableColumn id="2" name="Order"/>
+    <x:tableColumn id="3" name="Title"/>
+    <x:tableColumn id="4" name="Derived status"/>
+    <x:tableColumn id="5" name="Exit status"/>
+    <x:tableColumn id="6" name="Dependencies"/>
+    <x:tableColumn id="7" name="Completion workflows"/>
+    <x:tableColumn id="8" name="Primary findings"/>
+    <x:tableColumn id="9" name="Task selectors"/>
+    <x:tableColumn id="10" name="Target paths"/>
+    <x:tableColumn id="11" name="Launch gates"/>
+    <x:tableColumn id="12" name="Exit criteria"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AuditFindings" displayName="AuditFindings" ref="A1:M80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:M80"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Finding ID"/>
@@ -1937,8 +2077,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AuditWorkflows" displayName="AuditWorkflows" ref="A1:Q21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AuditWorkflows" displayName="AuditWorkflows" ref="A1:Q21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:Q21"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Workflow ID"/>
@@ -1963,8 +2103,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AuditSpecTasks" displayName="AuditSpecTasks" ref="A1:J363" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AuditSpecTasks" displayName="AuditSpecTasks" ref="A1:J363" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:J363"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Task ID"/>
@@ -1977,25 +2117,6 @@
     <x:tableColumn id="8" name="Workflows"/>
     <x:tableColumn id="9" name="Blockers"/>
     <x:tableColumn id="10" name="Prior claims"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AuditLaunchGates" displayName="AuditLaunchGates" ref="A1:J19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J19"/>
-  <x:tableColumns count="10">
-    <x:tableColumn id="1" name="Gate ID"/>
-    <x:tableColumn id="2" name="Title"/>
-    <x:tableColumn id="3" name="Wave"/>
-    <x:tableColumn id="4" name="Check kind"/>
-    <x:tableColumn id="5" name="Command"/>
-    <x:tableColumn id="6" name="Acceptance"/>
-    <x:tableColumn id="7" name="Evidence kinds"/>
-    <x:tableColumn id="8" name="Dependencies"/>
-    <x:tableColumn id="9" name="Owner"/>
-    <x:tableColumn id="10" name="Evidence status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2224,7 +2345,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="17" t="str">
-        <x:v>Canonical registry v7 • baseline codex/admin-workflow-completion@a043d35d4304 • source e1cccbdab5c7</x:v>
+        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 90d02de949e7</x:v>
       </x:c>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
@@ -3025,61 +3146,1266 @@
     <x:mergeCell ref="I19:J19"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:A5">
-    <x:cfRule type="expression" dxfId="54" priority="1">
+    <x:cfRule type="expression" dxfId="63" priority="1">
       <x:formula>A5="NO-GO"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C14:C31">
-    <x:cfRule type="containsText" dxfId="55" priority="2" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="56" priority="3" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="57" priority="4" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="58" priority="5" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="59" priority="6" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="60" priority="7" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="61" priority="8" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="62" priority="9" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="63" priority="10" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="64" priority="2" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="65" priority="3" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="66" priority="4" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="67" priority="5" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="68" priority="6" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="69" priority="7" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="70" priority="8" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="71" priority="9" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="72" priority="10" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F14:F20">
-    <x:cfRule type="containsText" dxfId="64" priority="11" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="65" priority="12" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="66" priority="13" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="67" priority="14" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="68" priority="15" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="69" priority="16" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="70" priority="17" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="71" priority="18" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="72" priority="19" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="73" priority="11" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="74" priority="12" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="75" priority="13" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="76" priority="14" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="77" priority="15" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="78" priority="16" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="79" priority="17" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="80" priority="18" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="81" priority="19" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F24:F30">
-    <x:cfRule type="containsText" dxfId="73" priority="20" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="74" priority="21" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="75" priority="22" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="76" priority="23" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="77" priority="24" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="78" priority="25" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="79" priority="26" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="80" priority="27" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="81" priority="28" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="82" priority="20" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="83" priority="21" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="84" priority="22" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="85" priority="23" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="86" priority="24" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="87" priority="25" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="88" priority="26" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="89" priority="27" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="90" priority="28" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="I14:I17">
-    <x:cfRule type="containsText" dxfId="82" priority="29" operator="containsText" text="P0"/>
-    <x:cfRule type="containsText" dxfId="83" priority="30" operator="containsText" text="P1"/>
-    <x:cfRule type="containsText" dxfId="84" priority="31" operator="containsText" text="P2"/>
-    <x:cfRule type="containsText" dxfId="85" priority="32" operator="containsText" text="P3"/>
+    <x:cfRule type="containsText" dxfId="91" priority="29" operator="containsText" text="P0"/>
+    <x:cfRule type="containsText" dxfId="92" priority="30" operator="containsText" text="P1"/>
+    <x:cfRule type="containsText" dxfId="93" priority="31" operator="containsText" text="P2"/>
+    <x:cfRule type="containsText" dxfId="94" priority="32" operator="containsText" text="P3"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e176c6fc9184a81"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R707201d78ef44d85"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4887867c656842e1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R220c144099f9406c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3577ede251db4bd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1383153fd30f46e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R588ac78b110c4140"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5e016c94d584495"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a7e4c7e96234259"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae89837f8fb944d3"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="54" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>File</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="str">
+        <x:v>Disposition</x:v>
+      </x:c>
+      <x:c r="C1" s="9" t="str">
+        <x:v>Workflow</x:v>
+      </x:c>
+      <x:c r="D1" s="9" t="str">
+        <x:v>Finding</x:v>
+      </x:c>
+      <x:c r="E1" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="F1" s="9" t="str">
+        <x:v>Reviewed at</x:v>
+      </x:c>
+      <x:c r="G1" s="9" t="str">
+        <x:v>Required remediation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="44" customHeight="1">
+      <x:c r="A2" s="10" t="str">
+        <x:v>app/api/accounts/check-slug/route.ts</x:v>
+      </x:c>
+      <x:c r="B2" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C2" s="10" t="str">
+        <x:v>ADM-WF-018</x:v>
+      </x:c>
+      <x:c r="D2" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E2" s="10" t="str">
+        <x:v>identity-platform</x:v>
+      </x:c>
+      <x:c r="F2" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G2" s="10" t="str">
+        <x:v>Slug availability needs a narrow authenticated lookup RPC instead of a general privileged client.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="44" customHeight="1">
+      <x:c r="A3" s="10" t="str">
+        <x:v>app/api/events/[id]/claim/route.ts</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>ADM-WF-003</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>ADM-M-004</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>event-platform</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>Claim creation and auto-verification must move to the canonical event command with actor binding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="44" customHeight="1">
+      <x:c r="A4" s="10" t="str">
+        <x:v>app/api/events/[id]/tour/route.ts</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
+        <x:v>ADM-WF-005</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="str">
+        <x:v>ADM-M-004</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>tour-platform</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G4" s="10" t="str">
+        <x:v>Legacy event-to-tour writes must be replaced by the canonical events_v2 assignment command.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" s="10" t="str">
+        <x:v>app/api/groups/threads/[id]/messages/[messageId]/reactions/route.ts</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="str">
+        <x:v>ADM-WF-011</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="str">
+        <x:v>communications</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G5" s="10" t="str">
+        <x:v>Reaction writes should run as the authenticated member so thread membership RLS remains authoritative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="44" customHeight="1">
+      <x:c r="A6" s="10" t="str">
+        <x:v>app/api/marketplace/admin/fee-rules/route.ts</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="str">
+        <x:v>Platform fee administration requires a named internal module, audit events, and bounded authority.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="A7" s="10" t="str">
+        <x:v>app/api/marketplace/admin/moderation/route.ts</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F7" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G7" s="10" t="str">
+        <x:v>Marketplace moderation is platform-internal and needs a reviewed module with explicit actor attribution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="A8" s="10" t="str">
+        <x:v>app/api/marketplace/admin/overview/route.ts</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F8" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="str">
+        <x:v>The internal marketplace overview must use a bounded read module instead of a bare privileged client.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="A9" s="10" t="str">
+        <x:v>app/api/marketplace/admin/webhook-events/route.ts</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F9" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="str">
+        <x:v>Webhook replay and inspection require an internal reviewed job with idempotency and audit evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="44" customHeight="1">
+      <x:c r="A10" s="10" t="str">
+        <x:v>app/api/marketplace/checkout/route.ts</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F10" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="str">
+        <x:v>Checkout orchestration needs a named transactional module with target validation and durable idempotency.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="44" customHeight="1">
+      <x:c r="A11" s="10" t="str">
+        <x:v>app/api/marketplace/order/[token]/claim/route.ts</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F11" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G11" s="10" t="str">
+        <x:v>Token claim must be an atomic token-bound RPC that cannot expose or mutate unrelated orders.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="44" customHeight="1">
+      <x:c r="A12" s="10" t="str">
+        <x:v>app/api/marketplace/order/[token]/route.ts</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F12" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="str">
+        <x:v>Public order lookup needs a minimal token-bound projection rather than unrestricted table access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="44" customHeight="1">
+      <x:c r="A13" s="10" t="str">
+        <x:v>app/api/ticketing/events/[eventId]/invites/[inviteId]/[action]/route.ts</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>ticketing</x:v>
+      </x:c>
+      <x:c r="F13" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G13" s="10" t="str">
+        <x:v>Invite lifecycle actions should be actor-bound transactional commands with event organization checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="44" customHeight="1">
+      <x:c r="A14" s="10" t="str">
+        <x:v>app/api/ticketing/events/[eventId]/sales-orders/route.ts</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>ticketing</x:v>
+      </x:c>
+      <x:c r="F14" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G14" s="10" t="str">
+        <x:v>Sales-order commands need a named ticketing module with verified event scope and audit attribution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="44" customHeight="1">
+      <x:c r="A15" s="10" t="str">
+        <x:v>app/api/tours/invitations/[token]/route.ts</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>ADM-WF-005</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>tour-platform</x:v>
+      </x:c>
+      <x:c r="F15" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G15" s="10" t="str">
+        <x:v>Invitation preview and expiration need token-bound projections while acceptance stays actor-bound.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="44" customHeight="1">
+      <x:c r="A16" s="10" t="str">
+        <x:v>app/api/venue/equipment/route.ts</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>ADM-WF-010</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>venue-operations</x:v>
+      </x:c>
+      <x:c r="F16" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str">
+        <x:v>Venue equipment reads and writes should execute as the authenticated venue member under RLS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="44" customHeight="1">
+      <x:c r="A17" s="10" t="str">
+        <x:v>app/api/venue/finances/route.ts</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>ADM-WF-014</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="str">
+        <x:v>ADM-M-032</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="str">
+        <x:v>finance</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G17" s="10" t="str">
+        <x:v>Venue finance must become read-only for organization users and use authenticated scoped reads.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="A18" s="10" t="str">
+        <x:v>app/api/venue/shifts/requests/route.ts</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>ADM-WF-008</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>workforce</x:v>
+      </x:c>
+      <x:c r="F18" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G18" s="10" t="str">
+        <x:v>Shift request decisions must preserve the authenticated venue actor and tenant RLS boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="44" customHeight="1">
+      <x:c r="A19" s="10" t="str">
+        <x:v>app/api/venue/shifts/swaps/route.ts</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>ADM-WF-008</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>workforce</x:v>
+      </x:c>
+      <x:c r="F19" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G19" s="10" t="str">
+        <x:v>Shift swap operations should use authenticated membership policies and validated state transitions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="44" customHeight="1">
+      <x:c r="A20" s="10" t="str">
+        <x:v>app/api/venues/[id]/reviews/route.ts</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>ADM-WF-010</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="str">
+        <x:v>ADM-M-008</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>venue-platform</x:v>
+      </x:c>
+      <x:c r="F20" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="str">
+        <x:v>Review reads and writes should use public or authenticated policies without privileged global access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="44" customHeight="1">
+      <x:c r="A21" s="10" t="str">
+        <x:v>app/api/workforce/requests/notify/route.ts</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>ADM-WF-012</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
+        <x:v>ADM-M-063</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="str">
+        <x:v>workforce-delivery</x:v>
+      </x:c>
+      <x:c r="F21" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G21" s="10" t="str">
+        <x:v>Workforce notifications require a named delivery job with recipient validation and retry evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="44" customHeight="1">
+      <x:c r="A22" s="10" t="str">
+        <x:v>app/marketplace/order/[token]/page.tsx</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G22" s="10" t="str">
+        <x:v>The public order page needs a minimal token projection and must not instantiate a privileged client.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="44" customHeight="1">
+      <x:c r="A23" s="10" t="str">
+        <x:v>lib/rebuild/workforce-activity-notify.ts</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>ADM-WF-012</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
+        <x:v>ADM-M-063</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>workforce-delivery</x:v>
+      </x:c>
+      <x:c r="F23" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G23" s="10" t="str">
+        <x:v>Activity delivery must run as a named outbox job with organization scope and bounded retries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="44" customHeight="1">
+      <x:c r="A24" s="10" t="str">
+        <x:v>lib/ticketing/guest-list.server.ts</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>ticketing</x:v>
+      </x:c>
+      <x:c r="F24" s="13" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="str">
+        <x:v>Guest-list administration needs reviewed ticketing commands with event scope and actor attribution.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="B2:B24">
+    <x:cfRule type="containsText" dxfId="60" priority="1" operator="containsText" text="migrate_to_job"/>
+    <x:cfRule type="containsText" dxfId="61" priority="2" operator="containsText" text="replace_with_rpc"/>
+    <x:cfRule type="containsText" dxfId="62" priority="3" operator="containsText" text="replace_with_user_rls"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8317c41030a44717"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="44" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="54" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="68" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>Batch ID</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="str">
+        <x:v>Order</x:v>
+      </x:c>
+      <x:c r="C1" s="9" t="str">
+        <x:v>Title</x:v>
+      </x:c>
+      <x:c r="D1" s="9" t="str">
+        <x:v>Derived status</x:v>
+      </x:c>
+      <x:c r="E1" s="9" t="str">
+        <x:v>Exit status</x:v>
+      </x:c>
+      <x:c r="F1" s="9" t="str">
+        <x:v>Dependencies</x:v>
+      </x:c>
+      <x:c r="G1" s="9" t="str">
+        <x:v>Completion workflows</x:v>
+      </x:c>
+      <x:c r="H1" s="9" t="str">
+        <x:v>Primary findings</x:v>
+      </x:c>
+      <x:c r="I1" s="9" t="str">
+        <x:v>Task selectors</x:v>
+      </x:c>
+      <x:c r="J1" s="9" t="str">
+        <x:v>Target paths</x:v>
+      </x:c>
+      <x:c r="K1" s="9" t="str">
+        <x:v>Launch gates</x:v>
+      </x:c>
+      <x:c r="L1" s="9" t="str">
+        <x:v>Exit criteria</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="52" customHeight="1">
+      <x:c r="A2" s="10" t="str">
+        <x:v>ADM-B00</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C2" s="10" t="str">
+        <x:v>Execution control plane</x:v>
+      </x:c>
+      <x:c r="D2" s="10" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="E2" s="10" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="F2" s="10" t="str"/>
+      <x:c r="G2" s="10" t="str"/>
+      <x:c r="H2" s="10" t="str">
+        <x:v>AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+      </x:c>
+      <x:c r="I2" s="10" t="str"/>
+      <x:c r="J2" s="10" t="str">
+        <x:v>docs/admin-audit; scripts/audit; lib/admin/audit-registry-contracts.ts; package.json</x:v>
+      </x:c>
+      <x:c r="K2" s="10" t="str">
+        <x:v>LG-04</x:v>
+      </x:c>
+      <x:c r="L2" s="10" t="str">
+        <x:v>Every finding, specification task, and workflow completion has exactly one primary batch.; The generated ADM-B00 context pack is at most 32 KiB and all generated views have zero drift.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="52" customHeight="1">
+      <x:c r="A3" s="10" t="str">
+        <x:v>ADM-B01</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="str">
+        <x:v>Reproducible baseline and migration chain</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="str">
+        <x:v>blocked</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>ADM-B00</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str"/>
+      <x:c r="H3" s="10" t="str">
+        <x:v>ADM-M-001; ADM-M-010; ADM-M-013; ADM-M-058; ADM-M-061; AOA-003; AOA-012; AOA-015</x:v>
+      </x:c>
+      <x:c r="I3" s="10" t="str">
+        <x:v>^REL-(00[1-8]|10[1-4])$; SEC-005</x:v>
+      </x:c>
+      <x:c r="J3" s="10" t="str">
+        <x:v>supabase/migrations; scripts/ci; __tests__/admin; package.json</x:v>
+      </x:c>
+      <x:c r="K3" s="10" t="str">
+        <x:v>LG-01; LG-02; LG-03; LG-04; LG-05; LG-06</x:v>
+      </x:c>
+      <x:c r="L3" s="10" t="str">
+        <x:v>A fresh isolated database and representative legacy upgrade complete with reconciliation evidence.; The complete baseline command is repeatable and has no unexplained failures.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="52" customHeight="1">
+      <x:c r="A4" s="10" t="str">
+        <x:v>ADM-B02</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
+        <x:v>Identity, tenant isolation, and privileged execution</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="str">
+        <x:v>blocked</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="str">
+        <x:v>ADM-B01</x:v>
+      </x:c>
+      <x:c r="G4" s="10" t="str">
+        <x:v>ADM-WF-001; ADM-WF-002</x:v>
+      </x:c>
+      <x:c r="H4" s="10" t="str">
+        <x:v>ADM-M-002; ADM-M-003; ADM-M-006; ADM-M-012; ADM-M-016; ADM-M-017; ADM-M-018; ADM-M-019; ADM-M-021; ADM-M-047; ADM-M-051; ADM-M-052; ADM-M-053; ADM-M-054; ADM-M-055; ADM-M-056; ADM-M-057</x:v>
+      </x:c>
+      <x:c r="I4" s="10" t="str">
+        <x:v>^SEC-(00[1-4]|10[1-3]|10[5-9]|11[0-2]|20[1-5]|60[1-5])$; ^ADR-(001|002|003|009)$</x:v>
+      </x:c>
+      <x:c r="J4" s="10" t="str">
+        <x:v>lib/auth; lib/admin/api-route-registry.ts; app/api/admin; supabase/migrations; __tests__/admin/rls-persona-matrix.test.ts</x:v>
+      </x:c>
+      <x:c r="K4" s="10" t="str">
+        <x:v>LG-09; LG-11; LG-15</x:v>
+      </x:c>
+      <x:c r="L4" s="10" t="str">
+        <x:v>Org A, Org B, revoked, stale, unauthenticated, and technical-principal tests pass through API and direct data access.; No critical elevation, actor-binding, or tenant-isolation finding remains open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52" customHeight="1">
+      <x:c r="A5" s="10" t="str">
+        <x:v>ADM-B03</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="str">
+        <x:v>SEC-104 site-map zone recovery</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F5" s="10" t="str">
+        <x:v>ADM-B02</x:v>
+      </x:c>
+      <x:c r="G5" s="10" t="str"/>
+      <x:c r="H5" s="10" t="str"/>
+      <x:c r="I5" s="10" t="str">
+        <x:v>^MAP-; SEC-104</x:v>
+      </x:c>
+      <x:c r="J5" s="10" t="str">
+        <x:v>app/api/admin/logistics/site-maps; lib/admin/site-map-zones.ts; lib/site-map; supabase/migrations/20260903120000_site_map_zone_security_and_canonical_bridge.sql; __tests__/admin/site-map-*</x:v>
+      </x:c>
+      <x:c r="K5" s="10" t="str">
+        <x:v>LG-06; LG-11</x:v>
+      </x:c>
+      <x:c r="L5" s="10" t="str">
+        <x:v>Site-map zone collection and item commands enforce acting organization, capability, ownership, idempotency, and audit behavior.; Fresh migration, reconciliation, direct RLS bypass, retry, and recovery evidence passes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
+      <x:c r="A6" s="10" t="str">
+        <x:v>ADM-B04</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Canonical events and ingestion</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="str">
+        <x:v>ADM-B02</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="str">
+        <x:v>ADM-WF-003; ADM-WF-004</x:v>
+      </x:c>
+      <x:c r="H6" s="10" t="str">
+        <x:v>ADM-M-004; ADM-M-009; ADM-M-036</x:v>
+      </x:c>
+      <x:c r="I6" s="10" t="str">
+        <x:v>^EVENT-; ADR-004</x:v>
+      </x:c>
+      <x:c r="J6" s="10" t="str">
+        <x:v>app/api/admin/events; lib/admin/event-access.service.ts; supabase/migrations; __tests__/admin/event-*</x:v>
+      </x:c>
+      <x:c r="K6" s="10" t="str">
+        <x:v>LG-10; LG-14</x:v>
+      </x:c>
+      <x:c r="L6" s="10" t="str">
+        <x:v>Legacy event writes are retired and ID reconciliation reports zero unexplained discrepancies.; Provider ingestion through Admin publication passes with retry, rollback, and audit evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
+      <x:c r="A7" s="10" t="str">
+        <x:v>ADM-B05</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Tours and Artist delivery</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F7" s="10" t="str">
+        <x:v>ADM-B04</x:v>
+      </x:c>
+      <x:c r="G7" s="10" t="str">
+        <x:v>ADM-WF-005; ADM-WF-006</x:v>
+      </x:c>
+      <x:c r="H7" s="10" t="str">
+        <x:v>ADM-M-005; ADM-M-022; ADM-M-023; ADM-M-024; ADM-M-025; ADM-M-026; ADM-M-027; ADM-M-028</x:v>
+      </x:c>
+      <x:c r="I7" s="10" t="str">
+        <x:v>^(TOUR|PLAN|PUB)-; ADR-005; ADR-006</x:v>
+      </x:c>
+      <x:c r="J7" s="10" t="str">
+        <x:v>app/api/admin/tours; lib/admin/tour-access.service.ts; lib/admin/publication-*; components/admin; __tests__/admin/tour-*</x:v>
+      </x:c>
+      <x:c r="K7" s="10" t="str">
+        <x:v>LG-13; LG-14</x:v>
+      </x:c>
+      <x:c r="L7" s="10" t="str">
+        <x:v>Provider event to published tour to Artist-visible itinerary succeeds with canonical IDs and local-time correctness.; Autosave, duplicate, quarantine, holds, ghost-stop, idempotency, and recovery cases pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
+      <x:c r="A8" s="10" t="str">
+        <x:v>ADM-B06</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Hiring and onboarding</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="str">
+        <x:v>ADM-B02</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="str">
+        <x:v>ADM-WF-007</x:v>
+      </x:c>
+      <x:c r="H8" s="10" t="str">
+        <x:v>ADM-M-014; ADM-M-015; ADM-M-062</x:v>
+      </x:c>
+      <x:c r="I8" s="10" t="str">
+        <x:v>^HIRE-</x:v>
+      </x:c>
+      <x:c r="J8" s="10" t="str">
+        <x:v>app/api/admin/hiring; lib/hiring; components/hiring; supabase/migrations; __tests__/hiring</x:v>
+      </x:c>
+      <x:c r="K8" s="10" t="str">
+        <x:v>LG-12</x:v>
+      </x:c>
+      <x:c r="L8" s="10" t="str">
+        <x:v>Candidate invitation delivery, redemption, expiration, replay prevention, failure visibility, and organization scoping pass.; Accepted candidates provision exactly one worker identity and can continue to workforce assignment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="10" t="str">
+        <x:v>ADM-B07</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Workforce roster and check-in</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F9" s="10" t="str">
+        <x:v>ADM-B05; ADM-B06</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="str">
+        <x:v>ADM-WF-008</x:v>
+      </x:c>
+      <x:c r="H9" s="10" t="str">
+        <x:v>ADM-M-029</x:v>
+      </x:c>
+      <x:c r="I9" s="10" t="str">
+        <x:v>^WORK-</x:v>
+      </x:c>
+      <x:c r="J9" s="10" t="str">
+        <x:v>app/api/admin/workforce; lib/admin/workforce-*; components/hiring; __tests__/admin/workforce-*; __tests__/admin/check-in.test.ts</x:v>
+      </x:c>
+      <x:c r="K9" s="10" t="str">
+        <x:v>LG-12</x:v>
+      </x:c>
+      <x:c r="L9" s="10" t="str">
+        <x:v>Admin-to-worker assignment, notification, acknowledgement, roster, replacement, and check-in journeys pass.; Cross-organization, forged status, revoked user, duplicate, partial failure, and retry cases fail safely.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="10" t="str">
+        <x:v>ADM-B08</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>Messaging, private storage, and delivery workers</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="str">
+        <x:v>ADM-B02</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="str">
+        <x:v>ADM-WF-011; ADM-WF-012</x:v>
+      </x:c>
+      <x:c r="H10" s="10" t="str">
+        <x:v>ADM-M-011; ADM-M-020; ADM-M-030; ADM-M-031; ADM-M-064</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="str">
+        <x:v>^(COMMS|CAL)-</x:v>
+      </x:c>
+      <x:c r="J10" s="10" t="str">
+        <x:v>app/api/admin/communications; app/api/cron; lib/admin/comms-*; lib/admin/publication-outbox*; supabase/migrations; __tests__/admin/comms-*</x:v>
+      </x:c>
+      <x:c r="K10" s="10" t="str">
+        <x:v>LG-03; LG-11; LG-17</x:v>
+      </x:c>
+      <x:c r="L10" s="10" t="str">
+        <x:v>Private files reject public URLs and signed links expire or revoke as configured.; All scheduled workers expose idempotent retry, dead-letter, monitoring, and recipient delivery evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="52" customHeight="1">
+      <x:c r="A11" s="10" t="str">
+        <x:v>ADM-B09</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Operational logistics delivery</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="str">
+        <x:v>ADM-B03; ADM-B05; ADM-B07; ADM-B08</x:v>
+      </x:c>
+      <x:c r="G11" s="10" t="str">
+        <x:v>ADM-WF-013</x:v>
+      </x:c>
+      <x:c r="H11" s="10" t="str"/>
+      <x:c r="I11" s="10" t="str">
+        <x:v>^(ADV|LIVE|ROUTE|TRAVEL|TRANS|LODGE|LOG|EQUIP|RENT|CATER)-</x:v>
+      </x:c>
+      <x:c r="J11" s="10" t="str">
+        <x:v>app/api/admin/logistics; lib/admin/logistics-*; lib/admin/travel-*; components/admin/logistics; supabase/migrations; __tests__/admin/travel-*</x:v>
+      </x:c>
+      <x:c r="K11" s="10" t="str">
+        <x:v>LG-03; LG-11; LG-17</x:v>
+      </x:c>
+      <x:c r="L11" s="10" t="str">
+        <x:v>All operational records reference canonical event, stop, leg, organization, and recipient identities.; Producer, recipient acknowledgement, isolation, DST, partial failure, retry, and reversal journeys pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="52" customHeight="1">
+      <x:c r="A12" s="10" t="str">
+        <x:v>ADM-B10</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Organization, Artist, and Venue administration</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>ADM-B02</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="str">
+        <x:v>ADM-WF-009; ADM-WF-010; ADM-WF-018</x:v>
+      </x:c>
+      <x:c r="H12" s="10" t="str">
+        <x:v>ADM-M-007; ADM-M-008; ADM-M-045; ADM-M-046</x:v>
+      </x:c>
+      <x:c r="I12" s="10" t="str"/>
+      <x:c r="J12" s="10" t="str">
+        <x:v>app/admin/dashboard/artists; app/admin/dashboard/venues; app/admin/dashboard/organization; app/api/admin/artists; app/api/admin/venues; app/api/admin/organization</x:v>
+      </x:c>
+      <x:c r="K12" s="10" t="str">
+        <x:v>LG-11; LG-15</x:v>
+      </x:c>
+      <x:c r="L12" s="10" t="str">
+        <x:v>Search, CRUD, import, metrics, relationships, and deletion are tenant-scoped and server-authorized.; Org B, forged identifier, revoked user, direct API, and unsafe-delete tests pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="52" customHeight="1">
+      <x:c r="A13" s="10" t="str">
+        <x:v>ADM-B11</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Ticketing and admissions</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="str">
+        <x:v>ADM-B02; ADM-B04</x:v>
+      </x:c>
+      <x:c r="G13" s="10" t="str">
+        <x:v>ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="H13" s="10" t="str"/>
+      <x:c r="I13" s="10" t="str">
+        <x:v>^TIX-; ADR-007</x:v>
+      </x:c>
+      <x:c r="J13" s="10" t="str">
+        <x:v>app/api/admin/ticketing; lib/admin/ticketing-*; supabase/migrations; __tests__/admin/ticketing-*; __tests__/ticketing</x:v>
+      </x:c>
+      <x:c r="K13" s="10" t="str">
+        <x:v>LG-03; LG-11; LG-14</x:v>
+      </x:c>
+      <x:c r="L13" s="10" t="str">
+        <x:v>Ticketing producer-to-recipient and admissions journeys pass using canonical event identities.; Inventory, credential, device, webhook, offline, duplicate, isolation, and reconciliation cases pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="52" customHeight="1">
+      <x:c r="A14" s="10" t="str">
+        <x:v>ADM-B12</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Constrained commercial and provider administration</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>blocked</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F14" s="10" t="str">
+        <x:v>ADM-B02; ADM-B08</x:v>
+      </x:c>
+      <x:c r="G14" s="10" t="str">
+        <x:v>ADM-WF-014; ADM-WF-015; ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="H14" s="10" t="str">
+        <x:v>ADM-M-032; ADM-M-033; ADM-M-060; ADM-M-063</x:v>
+      </x:c>
+      <x:c r="I14" s="10" t="str">
+        <x:v>^(FIN|SETTLE|VEND|CONT)-; ADR-008</x:v>
+      </x:c>
+      <x:c r="J14" s="10" t="str">
+        <x:v>app/admin/dashboard/finances; app/admin/dashboard/contracts; app/api/admin/finance; app/api/admin/contracts; lib/admin/finance-*; lib/admin/contract-*</x:v>
+      </x:c>
+      <x:c r="K14" s="10" t="str">
+        <x:v>LG-03; LG-11; LG-17</x:v>
+      </x:c>
+      <x:c r="L14" s="10" t="str">
+        <x:v>Organization Admin finance writes, contract signing/executed claims, and provider tools are hidden and server-denied.; Allowed read, tracking, notification, export, isolation, and internal-platform journeys pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="52" customHeight="1">
+      <x:c r="A15" s="10" t="str">
+        <x:v>ADM-B13</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Navigation, accessibility, responsiveness, and reliability</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>ready_for_independent_verification</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="str">
+        <x:v>ADM-B05; ADM-B07; ADM-B08; ADM-B09; ADM-B10; ADM-B11; ADM-B12</x:v>
+      </x:c>
+      <x:c r="G15" s="10" t="str">
+        <x:v>ADM-WF-016</x:v>
+      </x:c>
+      <x:c r="H15" s="10" t="str">
+        <x:v>ADM-M-034; ADM-M-035; ADM-M-037; ADM-M-038; ADM-M-039; ADM-M-040; ADM-M-041; ADM-M-042; ADM-M-043; ADM-M-044; ADM-M-048; ADM-M-049; ADM-M-050; ADM-M-059</x:v>
+      </x:c>
+      <x:c r="I15" s="10" t="str">
+        <x:v>^(REP|EXP)-; ^REL-(201|202|301|401|501|60[1-4])$; ADR-010</x:v>
+      </x:c>
+      <x:c r="J15" s="10" t="str">
+        <x:v>app/admin/dashboard; components/admin; scripts/ci; tests/e2e; __tests__/admin/rel-phase6.test.ts</x:v>
+      </x:c>
+      <x:c r="K15" s="10" t="str">
+        <x:v>LG-16; LG-17</x:v>
+      </x:c>
+      <x:c r="L15" s="10" t="str">
+        <x:v>Critical journeys pass at phone, tablet, and desktop sizes using keyboard and screen-reader-oriented checks.; Navigation, query, performance, monitoring, retry, offline, and error-recovery budgets pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="52" customHeight="1">
+      <x:c r="A16" s="10" t="str">
+        <x:v>ADM-B14</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Independent verification and release</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="str">
+        <x:v>observed</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>done</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="str">
+        <x:v>ADM-B13</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="H16" s="10" t="str">
+        <x:v>AOA-007; AOA-013</x:v>
+      </x:c>
+      <x:c r="I16" s="10" t="str">
+        <x:v>^REL-(60[5-9]|61[01])$</x:v>
+      </x:c>
+      <x:c r="J16" s="10" t="str">
+        <x:v>docs/admin-audit; tests/e2e; scripts/ci; supabase/migrations</x:v>
+      </x:c>
+      <x:c r="K16" s="10" t="str">
+        <x:v>LG-01; LG-02; LG-03; LG-04; LG-05; LG-06; LG-07; LG-08; LG-09; LG-10; LG-11; LG-12; LG-13; LG-14; LG-15; LG-16; LG-17; LG-18</x:v>
+      </x:c>
+      <x:c r="L16" s="10" t="str">
+        <x:v>All required launch gates are evidence-complete on one immutable staging commit and a freshly migrated database.; Independent technical verification, product approval, security approval, and restricted pilot evidence are recorded with zero registry drift.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="D2:E16">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="evidence_complete"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e1ef1afb2664660"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5980,28 +7306,28 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="G2:G80">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="13" priority="5" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="14" priority="6" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="16" priority="8" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="17" priority="9" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C2:C80">
-    <x:cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="P0"/>
-    <x:cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="P1"/>
+    <x:cfRule type="containsText" dxfId="18" priority="10" operator="containsText" text="P0"/>
+    <x:cfRule type="containsText" dxfId="19" priority="11" operator="containsText" text="P1"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f669699e1a6457f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R437c4957864447d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7027,24 +8353,24 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="12" priority="2" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="14" priority="4" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="15" priority="5" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="16" priority="6" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="17" priority="7" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="18" priority="8" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="19" priority="9" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="21" priority="2" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="22" priority="3" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="23" priority="4" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="24" priority="5" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="25" priority="6" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="26" priority="7" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="27" priority="8" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="28" priority="9" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c45d33eac3d47a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7741937ee3134631"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -17978,24 +19304,24 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E2:E363">
-    <x:cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="21" priority="2" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="22" priority="3" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="23" priority="4" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="24" priority="5" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="25" priority="6" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="26" priority="7" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="27" priority="8" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="28" priority="9" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="29" priority="1" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="30" priority="2" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="31" priority="3" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="32" priority="4" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="33" priority="5" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="34" priority="6" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="35" priority="7" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="36" priority="8" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="37" priority="9" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e570dbb1aac4cdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd60d536012134bea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -18591,24 +19917,24 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J19">
-    <x:cfRule type="containsText" dxfId="29" priority="1" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="30" priority="2" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="31" priority="3" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="32" priority="4" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="33" priority="5" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="34" priority="6" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="35" priority="7" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="36" priority="8" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="37" priority="9" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="38" priority="1" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="40" priority="3" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="41" priority="4" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="42" priority="5" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="43" priority="6" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="44" priority="7" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="45" priority="8" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="46" priority="9" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3265ac6ec69d49e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4658d82a71cc427e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -18874,12 +20200,12 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F2:F7">
-    <x:cfRule type="containsText" dxfId="38" priority="2" operator="containsText" text="Critical"/>
-    <x:cfRule type="containsText" dxfId="39" priority="3" operator="containsText" text="High"/>
+    <x:cfRule type="containsText" dxfId="47" priority="2" operator="containsText" text="Critical"/>
+    <x:cfRule type="containsText" dxfId="48" priority="3" operator="containsText" text="High"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f71c7ea35864429"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad156f8b15424d1c"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -18900,7 +20226,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -19606,17 +20932,17 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C2:C19">
-    <x:cfRule type="containsText" dxfId="40" priority="1" operator="containsText" text="pass"/>
-    <x:cfRule type="containsText" dxfId="41" priority="2" operator="containsText" text="fail"/>
+    <x:cfRule type="containsText" dxfId="49" priority="1" operator="containsText" text="pass"/>
+    <x:cfRule type="containsText" dxfId="50" priority="2" operator="containsText" text="fail"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06bcd261c3964be3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b3b6e1837d741ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -19853,597 +21179,19 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F10">
-    <x:cfRule type="containsText" dxfId="42" priority="1" operator="containsText" text="done"/>
-    <x:cfRule type="containsText" dxfId="43" priority="2" operator="containsText" text="implemented"/>
-    <x:cfRule type="containsText" dxfId="44" priority="3" operator="containsText" text="ready_for_independent_verification"/>
-    <x:cfRule type="containsText" dxfId="45" priority="4" operator="containsText" text="ready_for_staging"/>
-    <x:cfRule type="containsText" dxfId="46" priority="5" operator="containsText" text="in_progress"/>
-    <x:cfRule type="containsText" dxfId="47" priority="6" operator="containsText" text="reproduced"/>
-    <x:cfRule type="containsText" dxfId="48" priority="7" operator="containsText" text="observed"/>
-    <x:cfRule type="containsText" dxfId="49" priority="8" operator="containsText" text="not_verified"/>
-    <x:cfRule type="containsText" dxfId="50" priority="9" operator="containsText" text="evidence_complete"/>
+    <x:cfRule type="containsText" dxfId="51" priority="1" operator="containsText" text="done"/>
+    <x:cfRule type="containsText" dxfId="52" priority="2" operator="containsText" text="implemented"/>
+    <x:cfRule type="containsText" dxfId="53" priority="3" operator="containsText" text="ready_for_independent_verification"/>
+    <x:cfRule type="containsText" dxfId="54" priority="4" operator="containsText" text="ready_for_staging"/>
+    <x:cfRule type="containsText" dxfId="55" priority="5" operator="containsText" text="in_progress"/>
+    <x:cfRule type="containsText" dxfId="56" priority="6" operator="containsText" text="reproduced"/>
+    <x:cfRule type="containsText" dxfId="57" priority="7" operator="containsText" text="observed"/>
+    <x:cfRule type="containsText" dxfId="58" priority="8" operator="containsText" text="not_verified"/>
+    <x:cfRule type="containsText" dxfId="59" priority="9" operator="containsText" text="evidence_complete"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b0dffc563e40e9"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="54" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="62" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="9" t="str">
-        <x:v>File</x:v>
-      </x:c>
-      <x:c r="B1" s="9" t="str">
-        <x:v>Disposition</x:v>
-      </x:c>
-      <x:c r="C1" s="9" t="str">
-        <x:v>Workflow</x:v>
-      </x:c>
-      <x:c r="D1" s="9" t="str">
-        <x:v>Finding</x:v>
-      </x:c>
-      <x:c r="E1" s="9" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="F1" s="9" t="str">
-        <x:v>Reviewed at</x:v>
-      </x:c>
-      <x:c r="G1" s="9" t="str">
-        <x:v>Required remediation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="44" customHeight="1">
-      <x:c r="A2" s="10" t="str">
-        <x:v>app/api/accounts/check-slug/route.ts</x:v>
-      </x:c>
-      <x:c r="B2" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C2" s="10" t="str">
-        <x:v>ADM-WF-018</x:v>
-      </x:c>
-      <x:c r="D2" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E2" s="10" t="str">
-        <x:v>identity-platform</x:v>
-      </x:c>
-      <x:c r="F2" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G2" s="10" t="str">
-        <x:v>Slug availability needs a narrow authenticated lookup RPC instead of a general privileged client.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="44" customHeight="1">
-      <x:c r="A3" s="10" t="str">
-        <x:v>app/api/events/[id]/claim/route.ts</x:v>
-      </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C3" s="10" t="str">
-        <x:v>ADM-WF-003</x:v>
-      </x:c>
-      <x:c r="D3" s="10" t="str">
-        <x:v>ADM-M-004</x:v>
-      </x:c>
-      <x:c r="E3" s="10" t="str">
-        <x:v>event-platform</x:v>
-      </x:c>
-      <x:c r="F3" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G3" s="10" t="str">
-        <x:v>Claim creation and auto-verification must move to the canonical event command with actor binding.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="44" customHeight="1">
-      <x:c r="A4" s="10" t="str">
-        <x:v>app/api/events/[id]/tour/route.ts</x:v>
-      </x:c>
-      <x:c r="B4" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C4" s="10" t="str">
-        <x:v>ADM-WF-005</x:v>
-      </x:c>
-      <x:c r="D4" s="10" t="str">
-        <x:v>ADM-M-004</x:v>
-      </x:c>
-      <x:c r="E4" s="10" t="str">
-        <x:v>tour-platform</x:v>
-      </x:c>
-      <x:c r="F4" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G4" s="10" t="str">
-        <x:v>Legacy event-to-tour writes must be replaced by the canonical events_v2 assignment command.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="44" customHeight="1">
-      <x:c r="A5" s="10" t="str">
-        <x:v>app/api/groups/threads/[id]/messages/[messageId]/reactions/route.ts</x:v>
-      </x:c>
-      <x:c r="B5" s="10" t="str">
-        <x:v>replace_with_user_rls</x:v>
-      </x:c>
-      <x:c r="C5" s="10" t="str">
-        <x:v>ADM-WF-011</x:v>
-      </x:c>
-      <x:c r="D5" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E5" s="10" t="str">
-        <x:v>communications</x:v>
-      </x:c>
-      <x:c r="F5" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G5" s="10" t="str">
-        <x:v>Reaction writes should run as the authenticated member so thread membership RLS remains authoritative.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="44" customHeight="1">
-      <x:c r="A6" s="10" t="str">
-        <x:v>app/api/marketplace/admin/fee-rules/route.ts</x:v>
-      </x:c>
-      <x:c r="B6" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C6" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D6" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E6" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F6" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G6" s="10" t="str">
-        <x:v>Platform fee administration requires a named internal module, audit events, and bounded authority.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="44" customHeight="1">
-      <x:c r="A7" s="10" t="str">
-        <x:v>app/api/marketplace/admin/moderation/route.ts</x:v>
-      </x:c>
-      <x:c r="B7" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C7" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D7" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E7" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F7" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G7" s="10" t="str">
-        <x:v>Marketplace moderation is platform-internal and needs a reviewed module with explicit actor attribution.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="44" customHeight="1">
-      <x:c r="A8" s="10" t="str">
-        <x:v>app/api/marketplace/admin/overview/route.ts</x:v>
-      </x:c>
-      <x:c r="B8" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C8" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D8" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F8" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G8" s="10" t="str">
-        <x:v>The internal marketplace overview must use a bounded read module instead of a bare privileged client.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="44" customHeight="1">
-      <x:c r="A9" s="10" t="str">
-        <x:v>app/api/marketplace/admin/webhook-events/route.ts</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C9" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D9" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E9" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F9" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G9" s="10" t="str">
-        <x:v>Webhook replay and inspection require an internal reviewed job with idempotency and audit evidence.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="44" customHeight="1">
-      <x:c r="A10" s="10" t="str">
-        <x:v>app/api/marketplace/checkout/route.ts</x:v>
-      </x:c>
-      <x:c r="B10" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C10" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D10" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E10" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F10" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G10" s="10" t="str">
-        <x:v>Checkout orchestration needs a named transactional module with target validation and durable idempotency.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="44" customHeight="1">
-      <x:c r="A11" s="10" t="str">
-        <x:v>app/api/marketplace/order/[token]/claim/route.ts</x:v>
-      </x:c>
-      <x:c r="B11" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C11" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D11" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E11" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F11" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G11" s="10" t="str">
-        <x:v>Token claim must be an atomic token-bound RPC that cannot expose or mutate unrelated orders.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="44" customHeight="1">
-      <x:c r="A12" s="10" t="str">
-        <x:v>app/api/marketplace/order/[token]/route.ts</x:v>
-      </x:c>
-      <x:c r="B12" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C12" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D12" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E12" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F12" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G12" s="10" t="str">
-        <x:v>Public order lookup needs a minimal token-bound projection rather than unrestricted table access.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="44" customHeight="1">
-      <x:c r="A13" s="10" t="str">
-        <x:v>app/api/ticketing/events/[eventId]/invites/[inviteId]/[action]/route.ts</x:v>
-      </x:c>
-      <x:c r="B13" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C13" s="10" t="str">
-        <x:v>ADM-WF-019</x:v>
-      </x:c>
-      <x:c r="D13" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E13" s="10" t="str">
-        <x:v>ticketing</x:v>
-      </x:c>
-      <x:c r="F13" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G13" s="10" t="str">
-        <x:v>Invite lifecycle actions should be actor-bound transactional commands with event organization checks.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="44" customHeight="1">
-      <x:c r="A14" s="10" t="str">
-        <x:v>app/api/ticketing/events/[eventId]/sales-orders/route.ts</x:v>
-      </x:c>
-      <x:c r="B14" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C14" s="10" t="str">
-        <x:v>ADM-WF-019</x:v>
-      </x:c>
-      <x:c r="D14" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E14" s="10" t="str">
-        <x:v>ticketing</x:v>
-      </x:c>
-      <x:c r="F14" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G14" s="10" t="str">
-        <x:v>Sales-order commands need a named ticketing module with verified event scope and audit attribution.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="44" customHeight="1">
-      <x:c r="A15" s="10" t="str">
-        <x:v>app/api/tours/invitations/[token]/route.ts</x:v>
-      </x:c>
-      <x:c r="B15" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C15" s="10" t="str">
-        <x:v>ADM-WF-005</x:v>
-      </x:c>
-      <x:c r="D15" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E15" s="10" t="str">
-        <x:v>tour-platform</x:v>
-      </x:c>
-      <x:c r="F15" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G15" s="10" t="str">
-        <x:v>Invitation preview and expiration need token-bound projections while acceptance stays actor-bound.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="44" customHeight="1">
-      <x:c r="A16" s="10" t="str">
-        <x:v>app/api/venue/equipment/route.ts</x:v>
-      </x:c>
-      <x:c r="B16" s="10" t="str">
-        <x:v>replace_with_user_rls</x:v>
-      </x:c>
-      <x:c r="C16" s="10" t="str">
-        <x:v>ADM-WF-010</x:v>
-      </x:c>
-      <x:c r="D16" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E16" s="10" t="str">
-        <x:v>venue-operations</x:v>
-      </x:c>
-      <x:c r="F16" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G16" s="10" t="str">
-        <x:v>Venue equipment reads and writes should execute as the authenticated venue member under RLS.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="44" customHeight="1">
-      <x:c r="A17" s="10" t="str">
-        <x:v>app/api/venue/finances/route.ts</x:v>
-      </x:c>
-      <x:c r="B17" s="10" t="str">
-        <x:v>replace_with_user_rls</x:v>
-      </x:c>
-      <x:c r="C17" s="10" t="str">
-        <x:v>ADM-WF-014</x:v>
-      </x:c>
-      <x:c r="D17" s="10" t="str">
-        <x:v>ADM-M-032</x:v>
-      </x:c>
-      <x:c r="E17" s="10" t="str">
-        <x:v>finance</x:v>
-      </x:c>
-      <x:c r="F17" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G17" s="10" t="str">
-        <x:v>Venue finance must become read-only for organization users and use authenticated scoped reads.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="44" customHeight="1">
-      <x:c r="A18" s="10" t="str">
-        <x:v>app/api/venue/shifts/requests/route.ts</x:v>
-      </x:c>
-      <x:c r="B18" s="10" t="str">
-        <x:v>replace_with_user_rls</x:v>
-      </x:c>
-      <x:c r="C18" s="10" t="str">
-        <x:v>ADM-WF-008</x:v>
-      </x:c>
-      <x:c r="D18" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E18" s="10" t="str">
-        <x:v>workforce</x:v>
-      </x:c>
-      <x:c r="F18" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G18" s="10" t="str">
-        <x:v>Shift request decisions must preserve the authenticated venue actor and tenant RLS boundary.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="44" customHeight="1">
-      <x:c r="A19" s="10" t="str">
-        <x:v>app/api/venue/shifts/swaps/route.ts</x:v>
-      </x:c>
-      <x:c r="B19" s="10" t="str">
-        <x:v>replace_with_user_rls</x:v>
-      </x:c>
-      <x:c r="C19" s="10" t="str">
-        <x:v>ADM-WF-008</x:v>
-      </x:c>
-      <x:c r="D19" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E19" s="10" t="str">
-        <x:v>workforce</x:v>
-      </x:c>
-      <x:c r="F19" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G19" s="10" t="str">
-        <x:v>Shift swap operations should use authenticated membership policies and validated state transitions.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="44" customHeight="1">
-      <x:c r="A20" s="10" t="str">
-        <x:v>app/api/venues/[id]/reviews/route.ts</x:v>
-      </x:c>
-      <x:c r="B20" s="10" t="str">
-        <x:v>replace_with_user_rls</x:v>
-      </x:c>
-      <x:c r="C20" s="10" t="str">
-        <x:v>ADM-WF-010</x:v>
-      </x:c>
-      <x:c r="D20" s="10" t="str">
-        <x:v>ADM-M-008</x:v>
-      </x:c>
-      <x:c r="E20" s="10" t="str">
-        <x:v>venue-platform</x:v>
-      </x:c>
-      <x:c r="F20" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G20" s="10" t="str">
-        <x:v>Review reads and writes should use public or authenticated policies without privileged global access.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="44" customHeight="1">
-      <x:c r="A21" s="10" t="str">
-        <x:v>app/api/workforce/requests/notify/route.ts</x:v>
-      </x:c>
-      <x:c r="B21" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C21" s="10" t="str">
-        <x:v>ADM-WF-012</x:v>
-      </x:c>
-      <x:c r="D21" s="10" t="str">
-        <x:v>ADM-M-063</x:v>
-      </x:c>
-      <x:c r="E21" s="10" t="str">
-        <x:v>workforce-delivery</x:v>
-      </x:c>
-      <x:c r="F21" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G21" s="10" t="str">
-        <x:v>Workforce notifications require a named delivery job with recipient validation and retry evidence.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="44" customHeight="1">
-      <x:c r="A22" s="10" t="str">
-        <x:v>app/marketplace/order/[token]/page.tsx</x:v>
-      </x:c>
-      <x:c r="B22" s="10" t="str">
-        <x:v>replace_with_rpc</x:v>
-      </x:c>
-      <x:c r="C22" s="10" t="str">
-        <x:v>ADM-WF-020</x:v>
-      </x:c>
-      <x:c r="D22" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E22" s="10" t="str">
-        <x:v>marketplace-platform</x:v>
-      </x:c>
-      <x:c r="F22" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G22" s="10" t="str">
-        <x:v>The public order page needs a minimal token projection and must not instantiate a privileged client.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="44" customHeight="1">
-      <x:c r="A23" s="10" t="str">
-        <x:v>lib/rebuild/workforce-activity-notify.ts</x:v>
-      </x:c>
-      <x:c r="B23" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C23" s="10" t="str">
-        <x:v>ADM-WF-012</x:v>
-      </x:c>
-      <x:c r="D23" s="10" t="str">
-        <x:v>ADM-M-063</x:v>
-      </x:c>
-      <x:c r="E23" s="10" t="str">
-        <x:v>workforce-delivery</x:v>
-      </x:c>
-      <x:c r="F23" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G23" s="10" t="str">
-        <x:v>Activity delivery must run as a named outbox job with organization scope and bounded retries.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="10" t="str">
-        <x:v>lib/ticketing/guest-list.server.ts</x:v>
-      </x:c>
-      <x:c r="B24" s="10" t="str">
-        <x:v>migrate_to_job</x:v>
-      </x:c>
-      <x:c r="C24" s="10" t="str">
-        <x:v>ADM-WF-019</x:v>
-      </x:c>
-      <x:c r="D24" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
-      </x:c>
-      <x:c r="E24" s="10" t="str">
-        <x:v>ticketing</x:v>
-      </x:c>
-      <x:c r="F24" s="13" t="n">
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G24" s="10" t="str">
-        <x:v>Guest-list administration needs reviewed ticketing commands with event scope and actor attribution.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:conditionalFormatting sqref="B2:B24">
-    <x:cfRule type="containsText" dxfId="51" priority="1" operator="containsText" text="migrate_to_job"/>
-    <x:cfRule type="containsText" dxfId="52" priority="2" operator="containsText" text="replace_with_rpc"/>
-    <x:cfRule type="containsText" dxfId="53" priority="3" operator="containsText" text="replace_with_user_rls"/>
-  </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb45f92ea9af540bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cca01d6e4624401"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(admin): record execution control evidence
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbb089974eab643ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="Rb20779da8c53452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="R800f2532a5934f8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R9c83015765fb4bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R4ee3b864f5524a0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="Rb4eeb0e239274aa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R7c90c056dcbd494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="Rb4aa602a9acc4d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R3d53a2fe7c56450e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="Rf7722bebe23042a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R078bfb671f6c4d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="R628f2df8d497457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="Rd5ebb690afb14edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R31f340ef18c9484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R64f503857a4749cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="R3c2adf6a34684b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="Rf2cb2c87e7af443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="R25d5583dbd5e4f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R41df445cd64e42ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="Rf92cbb486c904e60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1942,8 +1942,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditEvidence" displayName="AuditEvidence" ref="A1:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:L19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditEvidence" displayName="AuditEvidence" ref="A1:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L21"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Kind"/>
@@ -2345,7 +2345,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="17" t="str">
-        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 90d02de949e7</x:v>
+        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 9065506f6351</x:v>
       </x:c>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
@@ -2476,8 +2476,8 @@
       </x:c>
       <x:c r="D9" s="31"/>
       <x:c r="E9" s="94" t="n">
-        <x:f>COUNTIF('Evidence'!$C$2:$C$19,"pass")</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTIF('Evidence'!$C$2:$C$21,"pass")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F9" s="95"/>
       <x:c r="G9" s="110" t="n">
@@ -3191,11 +3191,11 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1383153fd30f46e4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R588ac78b110c4140"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5e016c94d584495"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a7e4c7e96234259"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae89837f8fb944d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redc75372011d4bbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6911a5a319114a1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74deb131badd49a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2b0d41b792844da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R033e2329a7d94d09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3773,7 +3773,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8317c41030a44717"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R804f6eebcd914bad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4400,7 +4400,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e1ef1afb2664660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6f6b6b078674923"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7322,7 +7322,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R437c4957864447d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24f41df53d2a4679"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8365,7 +8365,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7741937ee3134631"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1757bf296c534d2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19316,7 +19316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd60d536012134bea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7201b4a799ac4122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19929,7 +19929,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4658d82a71cc427e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb211fa9be594083"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20205,7 +20205,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad156f8b15424d1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bf3e3956e5f4db7"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -20284,7 +20284,7 @@
     </x:row>
     <x:row r="2" ht="46" customHeight="1">
       <x:c r="A2" s="10" t="str">
-        <x:v>EVD-BASELINE-CHECKPOINT</x:v>
+        <x:v>EVD-B00-EXECUTION-CONTROL-COMMIT</x:v>
       </x:c>
       <x:c r="B2" s="10" t="str">
         <x:v>commit</x:v>
@@ -20296,67 +20296,69 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E2" s="12" t="n">
-        <x:v>46261.39236111111</x:v>
+        <x:v>46270.88297453704</x:v>
       </x:c>
       <x:c r="F2" s="10" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex implementation session</x:v>
       </x:c>
       <x:c r="G2" s="10" t="str">
-        <x:v>a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
+        <x:v>59d951c0e1bc2a67b7cc0289ffabb7dc1ee1644d</x:v>
       </x:c>
       <x:c r="H2" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
+        <x:v>git commit 59d951c0e1bc2a67b7cc0289ffabb7dc1ee1644d</x:v>
       </x:c>
       <x:c r="I2" s="10" t="str">
-        <x:v>AOA-002; AOA-015</x:v>
+        <x:v>AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J2" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K2" s="10" t="str"/>
       <x:c r="L2" s="10" t="str">
-        <x:v>Immutable checkpoint of the 138-path August 21 workspace baseline. Human inventory sign-off remains a separate release control.</x:v>
+        <x:v>Immutable implementation checkpoint for the token-efficient Admin execution control plane. The earlier site-map WIP checkpoint receives no completion credit.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="46" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>EVD-SEC104-LOGISTICS-DDL-LOCAL-FAIL</x:v>
+        <x:v>EVD-B00-EXECUTION-CONTROL-LOCAL</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
         <x:v>test_run</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
-        <x:v>fail</x:v>
+        <x:v>pass</x:v>
       </x:c>
       <x:c r="D3" s="10" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="E3" s="12" t="n">
-        <x:v>46268.959027777775</x:v>
+        <x:v>46270.88297453704</x:v>
       </x:c>
       <x:c r="F3" s="10" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex implementation session</x:v>
       </x:c>
       <x:c r="G3" s="10" t="str">
-        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>59d951c0e1bc2a67b7cc0289ffabb7dc1ee1644d</x:v>
       </x:c>
       <x:c r="H3" s="10" t="str">
-        <x:v>npx vitest run __tests__/logistics/logistics-route-contract.test.ts</x:v>
+        <x:v>audit-artifacts/admin-execution/ADM-B00/01.log</x:v>
       </x:c>
       <x:c r="I3" s="10" t="str">
-        <x:v>ADM-M-010</x:v>
+        <x:v>AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J3" s="10" t="str">
-        <x:v>ADM-WF-013; ADM-WF-017</x:v>
-      </x:c>
-      <x:c r="K3" s="10" t="str"/>
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K3" s="10" t="str">
+        <x:v>LG-04</x:v>
+      </x:c>
       <x:c r="L3" s="10" t="str">
-        <x:v>Six contract assertions pass and three fail because logistics_team_communications_scope, logistics_ops_foundation, and site_map_zone_ownership exist only in the pre-reconciliation archive. The failure is retained as evidence of active migration-chain debt.</x:v>
+        <x:v>Focused ADM-B00 validation passed. Exact coverage is 79 findings, 362 specification tasks, 20 workflow completions, and 15 execution batches; every generated context pack is within 32 KiB.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="46" customHeight="1">
       <x:c r="A4" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ACTING-COMMIT</x:v>
+        <x:v>EVD-BASELINE-CHECKPOINT</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
         <x:v>commit</x:v>
@@ -20368,67 +20370,67 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>46262.35711805556</x:v>
+        <x:v>46261.39236111111</x:v>
       </x:c>
       <x:c r="F4" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G4" s="10" t="str">
-        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
+        <x:v>a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
       </x:c>
       <x:c r="H4" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
+        <x:v>git:codex/admin-workflow-completion@a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
       </x:c>
       <x:c r="I4" s="10" t="str">
-        <x:v>ADM-M-013; ADM-M-019</x:v>
+        <x:v>AOA-002; AOA-015</x:v>
       </x:c>
       <x:c r="J4" s="10" t="str">
-        <x:v>ADM-WF-013; ADM-WF-017</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K4" s="10" t="str"/>
       <x:c r="L4" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint binding linked site maps to the acting organization and replacing the generic activity writer with validated, actor-bound commands.</x:v>
+        <x:v>Immutable checkpoint of the 138-path August 21 workspace baseline. Human inventory sign-off remains a separate release control.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="46" customHeight="1">
       <x:c r="A5" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
+        <x:v>EVD-SEC104-LOGISTICS-DDL-LOCAL-FAIL</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
         <x:v>test_run</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>pass</x:v>
+        <x:v>fail</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>46262.35711805556</x:v>
+        <x:v>46268.959027777775</x:v>
       </x:c>
       <x:c r="F5" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G5" s="10" t="str">
-        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
+        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H5" s="10" t="str">
-        <x:v>Node 20 route registry, focused active-org/tamper/actor-binding tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
+        <x:v>npx vitest run __tests__/logistics/logistics-route-contract.test.ts</x:v>
       </x:c>
       <x:c r="I5" s="10" t="str">
-        <x:v>ADM-M-013; ADM-M-019</x:v>
+        <x:v>ADM-M-010</x:v>
       </x:c>
       <x:c r="J5" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K5" s="10" t="str"/>
       <x:c r="L5" s="10" t="str">
-        <x:v>Local verification passed: 288 routes at 113/113 legacy; linked Org A/Org B mismatch and unscoped-map denial; forged activity action/actor/status rejection; child-map ownership; 230 active Admin files and 3,218 active tests. Live RLS and staging remain unverified.</x:v>
+        <x:v>Six contract assertions pass and three fail because logistics_team_communications_scope, logistics_ops_foundation, and site_map_zone_ownership exist only in the pre-reconciliation archive. The failure is retained as evidence of active migration-chain debt.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COLLAB-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ACTING-COMMIT</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
         <x:v>commit</x:v>
@@ -20440,31 +20442,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>46262.3608912037</x:v>
+        <x:v>46262.35711805556</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G6" s="10" t="str">
-        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
+        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="H6" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
+        <x:v>git:codex/admin-workflow-completion@abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="I6" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K6" s="10" t="str"/>
       <x:c r="L6" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint migrating site-map collaborator reads/removals to active-org capabilities while preserving owner-only removal.</x:v>
+        <x:v>Immutable SEC-104 checkpoint binding linked site maps to the acting organization and replacing the generic activity writer with validated, actor-bound commands.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20476,31 +20478,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>46262.3608912037</x:v>
+        <x:v>46262.35711805556</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G7" s="10" t="str">
-        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
+        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="H7" s="10" t="str">
-        <x:v>Node 20 route registry, collaborator input/source tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
+        <x:v>Node 20 route registry, focused active-org/tamper/actor-binding tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K7" s="10" t="str"/>
       <x:c r="L7" s="10" t="str">
-        <x:v>Local verification passed: 288 routes at 112/112 legacy; strict collaborator UUID/tamper rejection; active-org plus owner-only removal boundary; 231 active Admin files and 3,223 active tests. Live RLS and staging remain unverified.</x:v>
+        <x:v>Local verification passed: 288 routes at 113/113 legacy; linked Org A/Org B mismatch and unscoped-map denial; forged activity action/actor/status rejection; child-map ownership; 230 active Admin files and 3,218 active tests. Live RLS and staging remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COLLAB-COMMIT</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
         <x:v>commit</x:v>
@@ -20512,16 +20514,16 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46262.3608912037</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G8" s="10" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="H8" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>git:codex/admin-workflow-completion@63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="I8" s="10" t="str">
         <x:v>ADM-M-013</x:v>
@@ -20531,15 +20533,15 @@
       </x:c>
       <x:c r="K8" s="10" t="str"/>
       <x:c r="L8" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map collaborator reads/removals to active-org capabilities while preserving owner-only removal.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>pass</x:v>
@@ -20548,34 +20550,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>46268.959027777775</x:v>
+        <x:v>46262.3608912037</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
-        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>Node 20 route registry, collaborator input/source tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I9" s="10" t="str">
-        <x:v>ADM-M-013; ADM-M-019</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K9" s="10" t="str"/>
       <x:c r="L9" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint for selected-organization-bound site-map element commands, actor-bound RLS, atomic canvas synchronization, database-side tamper constraints, canonical events_v2 parent resolution, and collaborator expiration.</x:v>
+        <x:v>Local verification passed: 288 routes at 112/112 legacy; strict collaborator UUID/tamper rejection; active-org plus owner-only removal boundary; 231 active Admin files and 3,223 active tests. Live RLS and staging remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
         <x:v>pass</x:v>
@@ -20584,34 +20586,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>46268.959027777775</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
-        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, scoped TypeScript, route registry, migration validation, service-role allowlist, and registry validation recorded in TASK_LOG.md</x:v>
+        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="I10" s="10" t="str">
-        <x:v>ADM-M-013; ADM-M-019</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K10" s="10" t="str"/>
       <x:c r="L10" s="10" t="str">
-        <x:v>Local verification passed: 30 focused tests; exact 288-route parity at 110/110 legacy; 233 Admin files and 3,244 Admin tests; touched lint and scoped TypeScript; migration and service-role controls. One live-security file and two environment-dependent Admin tests remain skipped.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-RLS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-COMMIT</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>rls_matrix</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>pass</x:v>
@@ -20629,7 +20631,7 @@
         <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>Disposable PostgreSQL fixture: migration apply plus owner, replay, cross-map collision, forged tenant field, invalid geometry, expired collaborator, rollback, cross-actor read, and cross-actor write assertions</x:v>
+        <x:v>git:codex/admin-workflow-completion@7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="I11" s="10" t="str">
         <x:v>ADM-M-013; ADM-M-019</x:v>
@@ -20639,12 +20641,12 @@
       </x:c>
       <x:c r="K11" s="10" t="str"/>
       <x:c r="L11" s="10" t="str">
-        <x:v>The migration parsed and applied to a fresh disposable local PostgreSQL schema. Atomic replay and rollback plus direct actor/tamper/expiry denials passed. This is isolated local evidence, not dedicated Supabase staging or a complete Org A/Org B matrix.</x:v>
+        <x:v>Immutable SEC-104 checkpoint for selected-organization-bound site-map element commands, actor-bound RLS, atomic canvas synchronization, database-side tamper constraints, canonical events_v2 parent resolution, and collaborator expiration.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-LOCAL</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20656,34 +20658,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E12" s="12" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46268.959027777775</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G12" s="10" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
+        <x:v>SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, scoped TypeScript, route registry, migration validation, service-role allowlist, and registry validation recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I12" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K12" s="10" t="str"/>
       <x:c r="L12" s="10" t="str">
-        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
+        <x:v>Local verification passed: 30 focused tests; exact 288-route parity at 110/110 legacy; 233 Admin files and 3,244 Admin tests; touched lint and scoped TypeScript; migration and service-role controls. One live-security file and two environment-dependent Admin tests remain skipped.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-RLS-LOCAL</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>rls_matrix</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
         <x:v>pass</x:v>
@@ -20692,31 +20694,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E13" s="12" t="n">
-        <x:v>46262.33998842593</x:v>
+        <x:v>46268.959027777775</x:v>
       </x:c>
       <x:c r="F13" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G13" s="10" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H13" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
+        <x:v>Disposable PostgreSQL fixture: migration apply plus owner, replay, cross-map collision, forged tenant field, invalid geometry, expired collaborator, rollback, cross-actor read, and cross-actor write assertions</x:v>
       </x:c>
       <x:c r="I13" s="10" t="str">
-        <x:v>AOA-012</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K13" s="10" t="str"/>
       <x:c r="L13" s="10" t="str">
-        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
+        <x:v>The migration parsed and applied to a fresh disposable local PostgreSQL schema. Atomic replay and rollback plus direct actor/tamper/expiry denials passed. This is isolated local evidence, not dedicated Supabase staging or a complete Org A/Org B matrix.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="10" t="str">
-        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20728,34 +20730,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E14" s="12" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G14" s="10" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H14" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
+        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I14" s="10" t="str">
-        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K14" s="10" t="str"/>
       <x:c r="L14" s="10" t="str">
-        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
+        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
         <x:v>pass</x:v>
@@ -20764,7 +20766,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E15" s="12" t="n">
-        <x:v>46262.33961805556</x:v>
+        <x:v>46262.33998842593</x:v>
       </x:c>
       <x:c r="F15" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20773,22 +20775,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H15" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
       </x:c>
       <x:c r="I15" s="10" t="str">
-        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
+        <x:v>AOA-012</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K15" s="10" t="str"/>
       <x:c r="L15" s="10" t="str">
-        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
+        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20809,25 +20811,25 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H16" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
       </x:c>
       <x:c r="I16" s="10" t="str">
-        <x:v>AOA-013; AOA-015</x:v>
+        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J16" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K16" s="10" t="str"/>
       <x:c r="L16" s="10" t="str">
-        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
         <x:v>pass</x:v>
@@ -20836,7 +20838,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E17" s="12" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.33961805556</x:v>
       </x:c>
       <x:c r="F17" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20845,22 +20847,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H17" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="I17" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K17" s="10" t="str"/>
       <x:c r="L17" s="10" t="str">
-        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20881,34 +20883,34 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H18" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
       </x:c>
       <x:c r="I18" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>AOA-013; AOA-015</x:v>
       </x:c>
       <x:c r="J18" s="10" t="str">
-        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K18" s="10" t="str"/>
       <x:c r="L18" s="10" t="str">
-        <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
+        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="A19" s="10" t="str">
-        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
         <x:v>test_run</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>fail</x:v>
+        <x:v>pass</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="E19" s="12" t="n">
-        <x:v>46262.33513888889</x:v>
+        <x:v>46262.339895833335</x:v>
       </x:c>
       <x:c r="F19" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20917,27 +20919,99 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H19" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
       </x:c>
       <x:c r="I19" s="10" t="str">
-        <x:v>ADM-M-001; AOA-003</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J19" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K19" s="10" t="str"/>
       <x:c r="L19" s="10" t="str">
+        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="46" customHeight="1">
+      <x:c r="A20" s="10" t="str">
+        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>pass</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="n">
+        <x:v>46262.339895833335</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H20" s="10" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+      </x:c>
+      <x:c r="I20" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="J20" s="10" t="str">
+        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+      </x:c>
+      <x:c r="K20" s="10" t="str"/>
+      <x:c r="L20" s="10" t="str">
+        <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="46" customHeight="1">
+      <x:c r="A21" s="10" t="str">
+        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>fail</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="n">
+        <x:v>46262.33513888889</x:v>
+      </x:c>
+      <x:c r="F21" s="10" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G21" s="10" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H21" s="10" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
+      </x:c>
+      <x:c r="I21" s="10" t="str">
+        <x:v>ADM-M-001; AOA-003</x:v>
+      </x:c>
+      <x:c r="J21" s="10" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K21" s="10" t="str"/>
+      <x:c r="L21" s="10" t="str">
         <x:v>Pinned Node 20 full-repository typecheck exited 2 after 2,652.36 seconds. It checked 7,456 files, used about 6.3 GB, and reported type/schema drift across Admin and non-Admin code; the captured command output contained 3,005 lines. LG-01 remains not verified and the production build was not attempted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C19">
+  <x:conditionalFormatting sqref="C2:C21">
     <x:cfRule type="containsText" dxfId="49" priority="1" operator="containsText" text="pass"/>
     <x:cfRule type="containsText" dxfId="50" priority="2" operator="containsText" text="fail"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b3b6e1837d741ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd141d00dc7a54717"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21191,7 +21265,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cca01d6e4624401"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51561d64af814f83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ci): validate private migration tables correctly
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R078bfb671f6c4d89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="R628f2df8d497457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="Rd5ebb690afb14edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R31f340ef18c9484c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R64f503857a4749cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="R3c2adf6a34684b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="Rf2cb2c87e7af443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="R25d5583dbd5e4f5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R41df445cd64e42ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="Rf92cbb486c904e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd40b8aa7afbc41f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="R336a8f6702d54c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="R070f29a05a324c00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R1d05decf8ed14cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R96d763d095134ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="Rad7eb04ebfab4fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R686565c7d5ae474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="Raca09ebf619b40ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R2c5f1f8ce9ba4b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="R3de3939c3d354798"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2345,7 +2345,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="17" t="str">
-        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 9065506f6351</x:v>
+        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 65704f3d26a6</x:v>
       </x:c>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
@@ -3191,11 +3191,11 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redc75372011d4bbd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6911a5a319114a1a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74deb131badd49a0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2b0d41b792844da"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R033e2329a7d94d09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac07e9a474d94dff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591a1118e30044e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R139f098b520f4c22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R480ede593c5649ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b390c73dd0f4026"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3773,7 +3773,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R804f6eebcd914bad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5390a8bb951f4de4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4400,7 +4400,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6f6b6b078674923"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c7487426128402e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7322,7 +7322,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24f41df53d2a4679"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd52157b072e841dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8365,7 +8365,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1757bf296c534d2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9298ac7af6dd49e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19316,7 +19316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7201b4a799ac4122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R636407f8d15c479f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19929,7 +19929,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb211fa9be594083"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf47e9b76a84b4a74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20205,7 +20205,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bf3e3956e5f4db7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cc429248b2e451d"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -21011,7 +21011,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd141d00dc7a54717"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc662ace99b574c48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21265,7 +21265,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51561d64af814f83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re197fa39fc1e46ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(orchestrator): complete local task wave 29
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6d3b585279cf4df5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="R2dcc667c5b6e4304"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="Raf2665442f784b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R27a44b0ca3c945b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R89b53dc96efd44e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="R8443afad454f46b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R01b6a3eb4bf942b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="R45ef54aacf1a450c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R0ce49e7745284ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="R63ffab40cd624dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb00205119aa74b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="Rb4523d8be93a46dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="Rbc78ad3c83b84b2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R97273a9140bb4539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="Re6e35b0ad00b4c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="Rfb87c52b9e5d4f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R7053344248514450"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="Rd58b42b9606a4c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R9262b1fdd4194421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="Rfc53821ebfff435b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1979,8 +1979,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AuditServiceRoleDebt" displayName="AuditServiceRoleDebt" ref="A1:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G24"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AuditServiceRoleDebt" displayName="AuditServiceRoleDebt" ref="A1:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G31"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="File"/>
     <x:tableColumn id="2" name="Disposition"/>
@@ -2345,7 +2345,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="17" t="str">
-        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 17e3c841be9e</x:v>
+        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 9968c31640df</x:v>
       </x:c>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
@@ -2481,8 +2481,8 @@
       </x:c>
       <x:c r="F9" s="95"/>
       <x:c r="G9" s="110" t="n">
-        <x:f>COUNTA('Service Role Debt'!$A$2:$A$24)</x:f>
-        <x:v>23</x:v>
+        <x:f>COUNTA('Service Role Debt'!$A$2:$A$31)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="H9" s="111"/>
       <x:c r="I9" s="62" t="n">
@@ -2815,8 +2815,8 @@
         <x:v>migrate_to_job</x:v>
       </x:c>
       <x:c r="J21" s="2" t="n">
-        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$24,I21)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$31,I21)</x:f>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
@@ -2846,8 +2846,8 @@
         <x:v>replace_with_user_rls</x:v>
       </x:c>
       <x:c r="J22" s="2" t="n">
-        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$24,I22)</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$31,I22)</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
@@ -2879,8 +2879,8 @@
         <x:v>replace_with_rpc</x:v>
       </x:c>
       <x:c r="J23" s="2" t="n">
-        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$24,I23)</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$31,I23)</x:f>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
@@ -2913,7 +2913,7 @@
         <x:v>retire</x:v>
       </x:c>
       <x:c r="J24" s="2" t="n">
-        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$24,I24)</x:f>
+        <x:f>COUNTIF('Service Role Debt'!$B$2:$B$31,I24)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3191,11 +3191,11 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56cb725713d3410e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R344e9c73a2594ce8"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R782642c5d2354cab"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9263d29d120445c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9442c06ccf943cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R375e073dae71485d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3be45271703d400a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbbb1f268b8a43d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7709b26517864155"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e8e9880f4984440"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3765,15 +3765,176 @@
         <x:v>Guest-list administration needs reviewed ticketing commands with event scope and actor attribution.</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="44" customHeight="1">
+      <x:c r="A25" s="10" t="str">
+        <x:v>app/api/marketplace/orders/[id]/cancel/route.ts</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C25" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D25" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E25" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G25" s="10" t="str">
+        <x:v>Order cancellation needs a named marketplace command with bounded order scope, audit attribution, and compensating payout writes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="44" customHeight="1">
+      <x:c r="A26" s="10" t="str">
+        <x:v>app/api/marketplace/orders/[id]/refund/route.ts</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>marketplace-platform</x:v>
+      </x:c>
+      <x:c r="F26" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str">
+        <x:v>Order refunds need a named marketplace command with bounded order scope, idempotent provider actions, and audit attribution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="44" customHeight="1">
+      <x:c r="A27" s="10" t="str">
+        <x:v>app/api/messages/[conversationId]/realtime/route.ts</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="str">
+        <x:v>ADM-WF-011</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="str">
+        <x:v>ADM-M-030</x:v>
+      </x:c>
+      <x:c r="E27" s="10" t="str">
+        <x:v>communications</x:v>
+      </x:c>
+      <x:c r="F27" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G27" s="10" t="str">
+        <x:v>Realtime presence and receipt writes should retain the authenticated participant and enforce conversation membership through RLS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="44" customHeight="1">
+      <x:c r="A28" s="10" t="str">
+        <x:v>app/api/music/share-message/route.ts</x:v>
+      </x:c>
+      <x:c r="B28" s="10" t="str">
+        <x:v>replace_with_user_rls</x:v>
+      </x:c>
+      <x:c r="C28" s="10" t="str">
+        <x:v>ADM-WF-011</x:v>
+      </x:c>
+      <x:c r="D28" s="10" t="str">
+        <x:v>ADM-M-030</x:v>
+      </x:c>
+      <x:c r="E28" s="10" t="str">
+        <x:v>music-communications</x:v>
+      </x:c>
+      <x:c r="F28" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G28" s="10" t="str">
+        <x:v>Music share messages should write as the authenticated sender so conversation membership and recipient isolation remain authoritative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="44" customHeight="1">
+      <x:c r="A29" s="10" t="str">
+        <x:v>app/api/photos/purchase/webhook/route.ts</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>ADM-WF-020</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E29" s="10" t="str">
+        <x:v>photos-commerce</x:v>
+      </x:c>
+      <x:c r="F29" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G29" s="10" t="str">
+        <x:v>Verified photo purchase events need a named receipt-processing job with durable idempotency, bounded fulfillment, and audit evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="44" customHeight="1">
+      <x:c r="A30" s="10" t="str">
+        <x:v>app/api/webhooks/supabase/notifications/route.ts</x:v>
+      </x:c>
+      <x:c r="B30" s="10" t="str">
+        <x:v>migrate_to_job</x:v>
+      </x:c>
+      <x:c r="C30" s="10" t="str">
+        <x:v>ADM-WF-012</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="str">
+        <x:v>ADM-M-031</x:v>
+      </x:c>
+      <x:c r="E30" s="10" t="str">
+        <x:v>notification-delivery</x:v>
+      </x:c>
+      <x:c r="F30" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G30" s="10" t="str">
+        <x:v>Notification webhook delivery needs a named outbox job with recipient validation, durable duplicate suppression, and bounded retries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="44" customHeight="1">
+      <x:c r="A31" s="10" t="str">
+        <x:v>lib/auth/agent-service.ts</x:v>
+      </x:c>
+      <x:c r="B31" s="10" t="str">
+        <x:v>replace_with_rpc</x:v>
+      </x:c>
+      <x:c r="C31" s="10" t="str">
+        <x:v>ADM-WF-001</x:v>
+      </x:c>
+      <x:c r="D31" s="10" t="str">
+        <x:v>ADM-M-013</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="str">
+        <x:v>identity-platform</x:v>
+      </x:c>
+      <x:c r="F31" s="13" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="G31" s="10" t="str">
+        <x:v>Agent credential lookup and audit attribution need a narrow server RPC instead of a generally privileged client boundary.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="B2:B24">
+  <x:conditionalFormatting sqref="B2:B31">
     <x:cfRule type="containsText" dxfId="60" priority="1" operator="containsText" text="migrate_to_job"/>
     <x:cfRule type="containsText" dxfId="61" priority="2" operator="containsText" text="replace_with_rpc"/>
     <x:cfRule type="containsText" dxfId="62" priority="3" operator="containsText" text="replace_with_user_rls"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R656bbafe902840e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35bd1d16226e41d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4400,7 +4561,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b6a06ec49b3413c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R718bff3010aa436e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7322,7 +7483,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc277fad4745247b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1ee9f7cabcc4936"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8365,7 +8526,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7be00c0df984a9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84fc86936e3c46ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19316,7 +19477,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf2c90528c374f05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e6bddd0922a49e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19929,7 +20090,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4739e2b47e73453a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb75033994ac4483a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20205,7 +20366,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb193fec8222a48ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc3975d981734548"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -21253,7 +21414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06a9d2e53f3e4e33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6381789c44d84879"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21737,7 +21898,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R671a5357f1cc4316"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4aedb16cc8247d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(wip): record beta-K2 admin-workflow worktree state (reconciliation safety net)
Park uncommitted local state before pushing codex/admin-workflow-completion
to origin so no work is lost during consolidation:
- admin-audit generated trackers (ADM-B00..B14 contexts, workbook manifest,
  STATUS) and 2026 evidence records
- __tests__/qa + workforce-presenters test updates
- docker/local + production Dockerfile, next.config.ts, package.json
- supabase/migrations edit (artist jobs collaboration extension)
- orchestration helper scripts (check-active-migration-chain, context/task/
  status/verify) and docs/DEVELOPMENT_WORKFLOW, docs/work-packets
- TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx regression
</commit_message>
<xml_diff>
--- a/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
+++ b/docs/admin-audit/generated/TOURIFY_ADMIN_WORKFLOW_TRACKER.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd40b8aa7afbc41f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="R336a8f6702d54c36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="R070f29a05a324c00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="R1d05decf8ed14cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R96d763d095134ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="Rad7eb04ebfab4fa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R686565c7d5ae474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="Raca09ebf619b40ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="R2c5f1f8ce9ba4b23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="R3de3939c3d354798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdc504836624349a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Batches" sheetId="2" r:id="Rb321fd7ca6624363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" r:id="R5376ed29fcaf4646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="4" r:id="Rd44e33a706094d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Tasks" sheetId="5" r:id="R55846f8407954c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Gates" sheetId="6" r:id="R7108279152104028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R95ee208da38c4f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="8" r:id="Rd5a8779610684006"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="Rfb3ff564b2e04173"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Role Debt" sheetId="10" r:id="R228a27f0e2ed4c25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1942,8 +1942,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditEvidence" displayName="AuditEvidence" ref="A1:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:L21"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditEvidence" displayName="AuditEvidence" ref="A1:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L22"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Kind"/>
@@ -2345,7 +2345,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="17" t="str">
-        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source 65704f3d26a6</x:v>
+        <x:v>Canonical registry v8 • baseline codex/admin-workflow-completion@a043d35d4304 • source a9d7d7878bb4</x:v>
       </x:c>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
@@ -2476,8 +2476,8 @@
       </x:c>
       <x:c r="D9" s="31"/>
       <x:c r="E9" s="94" t="n">
-        <x:f>COUNTIF('Evidence'!$C$2:$C$21,"pass")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF('Evidence'!$C$2:$C$22,"pass")</x:f>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F9" s="95"/>
       <x:c r="G9" s="110" t="n">
@@ -3191,11 +3191,11 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac07e9a474d94dff"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591a1118e30044e9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R139f098b520f4c22"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R480ede593c5649ec"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b390c73dd0f4026"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62e13a80b2344e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R614a9ac3d6c94f03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7b1fc250c1443f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6d94ef68a74302"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc381481ef7624ac2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3773,7 +3773,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5390a8bb951f4de4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R157ecf5e6d864e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4400,7 +4400,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c7487426128402e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96beac1c5ab44cae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7322,7 +7322,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd52157b072e841dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94fd52c2d6b34813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8365,7 +8365,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9298ac7af6dd49e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafa9115552ea4441"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19316,7 +19316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R636407f8d15c479f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R316fde49d75244b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19929,7 +19929,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf47e9b76a84b4a74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17f362fa0dc643a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20205,7 +20205,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cc429248b2e451d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfadf3628c04744"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -20358,10 +20358,10 @@
     </x:row>
     <x:row r="4" ht="46" customHeight="1">
       <x:c r="A4" s="10" t="str">
-        <x:v>EVD-BASELINE-CHECKPOINT</x:v>
+        <x:v>EVD-B01-FOCUSED-LOCAL</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
         <x:v>pass</x:v>
@@ -20370,106 +20370,104 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>46261.39236111111</x:v>
+        <x:v>46270.92537037037</x:v>
       </x:c>
       <x:c r="F4" s="10" t="str">
-        <x:v>Codex</x:v>
-      </x:c>
-      <x:c r="G4" s="10" t="str">
-        <x:v>a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
-      </x:c>
+        <x:v>Codex implementation session</x:v>
+      </x:c>
+      <x:c r="G4" s="10"/>
       <x:c r="H4" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
+        <x:v>docs/admin-audit/evidence/2026/EVD-B01-FOCUSED-LOCAL.md</x:v>
       </x:c>
       <x:c r="I4" s="10" t="str">
-        <x:v>AOA-002; AOA-015</x:v>
+        <x:v>ADM-M-010; ADM-M-013; ADM-M-061; AOA-003; AOA-012; AOA-015</x:v>
       </x:c>
       <x:c r="J4" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K4" s="10" t="str"/>
       <x:c r="L4" s="10" t="str">
-        <x:v>Immutable checkpoint of the 138-path August 21 workspace baseline. Human inventory sign-off remains a separate release control.</x:v>
+        <x:v>All four declared ADM-B01 focused checks passed locally. This receipt intentionally remains local and uncommitted; CI, staging, fresh migration, type-check, build, and live RLS evidence are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="46" customHeight="1">
       <x:c r="A5" s="10" t="str">
-        <x:v>EVD-SEC104-LOGISTICS-DDL-LOCAL-FAIL</x:v>
+        <x:v>EVD-BASELINE-CHECKPOINT</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>fail</x:v>
+        <x:v>pass</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>46268.959027777775</x:v>
+        <x:v>46261.39236111111</x:v>
       </x:c>
       <x:c r="F5" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G5" s="10" t="str">
-        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
       </x:c>
       <x:c r="H5" s="10" t="str">
-        <x:v>npx vitest run __tests__/logistics/logistics-route-contract.test.ts</x:v>
+        <x:v>git:codex/admin-workflow-completion@a043d35d4304cc8181078a17e2138c1f47baf199</x:v>
       </x:c>
       <x:c r="I5" s="10" t="str">
-        <x:v>ADM-M-010</x:v>
+        <x:v>AOA-002; AOA-015</x:v>
       </x:c>
       <x:c r="J5" s="10" t="str">
-        <x:v>ADM-WF-013; ADM-WF-017</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K5" s="10" t="str"/>
       <x:c r="L5" s="10" t="str">
-        <x:v>Six contract assertions pass and three fail because logistics_team_communications_scope, logistics_ops_foundation, and site_map_zone_ownership exist only in the pre-reconciliation archive. The failure is retained as evidence of active migration-chain debt.</x:v>
+        <x:v>Immutable checkpoint of the 138-path August 21 workspace baseline. Human inventory sign-off remains a separate release control.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ACTING-COMMIT</x:v>
+        <x:v>EVD-SEC104-LOGISTICS-DDL-LOCAL-FAIL</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
-        <x:v>pass</x:v>
+        <x:v>fail</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>46262.35711805556</x:v>
+        <x:v>46268.959027777775</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G6" s="10" t="str">
-        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
+        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H6" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
+        <x:v>npx vitest run __tests__/logistics/logistics-route-contract.test.ts</x:v>
       </x:c>
       <x:c r="I6" s="10" t="str">
-        <x:v>ADM-M-013; ADM-M-019</x:v>
+        <x:v>ADM-M-010</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K6" s="10" t="str"/>
       <x:c r="L6" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint binding linked site maps to the acting organization and replacing the generic activity writer with validated, actor-bound commands.</x:v>
+        <x:v>Six contract assertions pass and three fail because logistics_team_communications_scope, logistics_ops_foundation, and site_map_zone_ownership exist only in the pre-reconciliation archive. The failure is retained as evidence of active migration-chain debt.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ACTING-COMMIT</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>pass</x:v>
@@ -20487,7 +20485,7 @@
         <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="H7" s="10" t="str">
-        <x:v>Node 20 route registry, focused active-org/tamper/actor-binding tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
+        <x:v>git:codex/admin-workflow-completion@abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
         <x:v>ADM-M-013; ADM-M-019</x:v>
@@ -20497,15 +20495,15 @@
       </x:c>
       <x:c r="K7" s="10" t="str"/>
       <x:c r="L7" s="10" t="str">
-        <x:v>Local verification passed: 288 routes at 113/113 legacy; linked Org A/Org B mismatch and unscoped-map denial; forged activity action/actor/status rejection; child-map ownership; 230 active Admin files and 3,218 active tests. Live RLS and staging remain unverified.</x:v>
+        <x:v>Immutable SEC-104 checkpoint binding linked site maps to the acting organization and replacing the generic activity writer with validated, actor-bound commands.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COLLAB-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ACTING-LOCAL</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>pass</x:v>
@@ -20514,34 +20512,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>46262.3608912037</x:v>
+        <x:v>46262.35711805556</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G8" s="10" t="str">
-        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
+        <x:v>abcf56c864b402f5cd85ecbeea618c8fa7edf89e</x:v>
       </x:c>
       <x:c r="H8" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
+        <x:v>Node 20 route registry, focused active-org/tamper/actor-binding tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I8" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K8" s="10" t="str"/>
       <x:c r="L8" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint migrating site-map collaborator reads/removals to active-org capabilities while preserving owner-only removal.</x:v>
+        <x:v>Local verification passed: 288 routes at 113/113 legacy; linked Org A/Org B mismatch and unscoped-map denial; forged activity action/actor/status rejection; child-map ownership; 230 active Admin files and 3,218 active tests. Live RLS and staging remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COLLAB-COMMIT</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>pass</x:v>
@@ -20559,7 +20557,7 @@
         <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>Node 20 route registry, collaborator input/source tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
+        <x:v>git:codex/admin-workflow-completion@63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="I9" s="10" t="str">
         <x:v>ADM-M-013</x:v>
@@ -20569,15 +20567,15 @@
       </x:c>
       <x:c r="K9" s="10" t="str"/>
       <x:c r="L9" s="10" t="str">
-        <x:v>Local verification passed: 288 routes at 112/112 legacy; strict collaborator UUID/tamper rejection; active-org plus owner-only removal boundary; 231 active Admin files and 3,223 active tests. Live RLS and staging remain unverified.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map collaborator reads/removals to active-org capabilities while preserving owner-only removal.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COLLAB-LOCAL</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
         <x:v>pass</x:v>
@@ -20586,16 +20584,16 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46262.3608912037</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>63ff56bd8a9567b6d34599d9afefa1e21780f950</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>Node 20 route registry, collaborator input/source tests, complete Admin Vitest, touched ESLint, scoped TypeScript, and audit-registry checks recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I10" s="10" t="str">
         <x:v>ADM-M-013</x:v>
@@ -20605,12 +20603,12 @@
       </x:c>
       <x:c r="K10" s="10" t="str"/>
       <x:c r="L10" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
+        <x:v>Local verification passed: 288 routes at 112/112 legacy; strict collaborator UUID/tamper rejection; active-org plus owner-only removal boundary; 231 active Admin files and 3,223 active tests. Live RLS and staging remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-COMMIT</x:v>
+        <x:v>EVD-SEC104-SITEMAP-COMMIT</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
         <x:v>commit</x:v>
@@ -20622,34 +20620,34 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>46268.959027777775</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
+        <x:v>git:codex/admin-workflow-completion@c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="I11" s="10" t="str">
-        <x:v>ADM-M-013; ADM-M-019</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K11" s="10" t="str"/>
       <x:c r="L11" s="10" t="str">
-        <x:v>Immutable SEC-104 checkpoint for selected-organization-bound site-map element commands, actor-bound RLS, atomic canvas synchronization, database-side tamper constraints, canonical events_v2 parent resolution, and collaborator expiration.</x:v>
+        <x:v>Immutable SEC-104 checkpoint migrating site-map template, export, and version routes to the trusted logistics.view acting-context boundary and reducing the enforced legacy ceiling to 114.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-COMMIT</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
         <x:v>pass</x:v>
@@ -20667,7 +20665,7 @@
         <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, scoped TypeScript, route registry, migration validation, service-role allowlist, and registry validation recorded in TASK_LOG.md</x:v>
+        <x:v>git:codex/admin-workflow-completion@7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="I12" s="10" t="str">
         <x:v>ADM-M-013; ADM-M-019</x:v>
@@ -20677,15 +20675,15 @@
       </x:c>
       <x:c r="K12" s="10" t="str"/>
       <x:c r="L12" s="10" t="str">
-        <x:v>Local verification passed: 30 focused tests; exact 288-route parity at 110/110 legacy; 233 Admin files and 3,244 Admin tests; touched lint and scoped TypeScript; migration and service-role controls. One live-security file and two environment-dependent Admin tests remain skipped.</x:v>
+        <x:v>Immutable SEC-104 checkpoint for selected-organization-bound site-map element commands, actor-bound RLS, atomic canvas synchronization, database-side tamper constraints, canonical events_v2 parent resolution, and collaborator expiration.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-RLS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-LOCAL</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>rls_matrix</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
         <x:v>pass</x:v>
@@ -20703,7 +20701,7 @@
         <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H13" s="10" t="str">
-        <x:v>Disposable PostgreSQL fixture: migration apply plus owner, replay, cross-map collision, forged tenant field, invalid geometry, expired collaborator, rollback, cross-actor read, and cross-actor write assertions</x:v>
+        <x:v>SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, scoped TypeScript, route registry, migration validation, service-role allowlist, and registry validation recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I13" s="10" t="str">
         <x:v>ADM-M-013; ADM-M-019</x:v>
@@ -20713,15 +20711,15 @@
       </x:c>
       <x:c r="K13" s="10" t="str"/>
       <x:c r="L13" s="10" t="str">
-        <x:v>The migration parsed and applied to a fresh disposable local PostgreSQL schema. Atomic replay and rollback plus direct actor/tamper/expiry denials passed. This is isolated local evidence, not dedicated Supabase staging or a complete Org A/Org B matrix.</x:v>
+        <x:v>Local verification passed: 30 focused tests; exact 288-route parity at 110/110 legacy; 233 Admin files and 3,244 Admin tests; touched lint and scoped TypeScript; migration and service-role controls. One live-security file and two environment-dependent Admin tests remain skipped.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="10" t="str">
-        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-ELEMENTS-RLS-LOCAL</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>rls_matrix</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>pass</x:v>
@@ -20730,31 +20728,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E14" s="12" t="n">
-        <x:v>46262.3490625</x:v>
+        <x:v>46268.959027777775</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G14" s="10" t="str">
-        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
+        <x:v>7630a37ef395e147198a169e94fa888d2f3c7b19</x:v>
       </x:c>
       <x:c r="H14" s="10" t="str">
-        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
+        <x:v>Disposable PostgreSQL fixture: migration apply plus owner, replay, cross-map collision, forged tenant field, invalid geometry, expired collaborator, rollback, cross-actor read, and cross-actor write assertions</x:v>
       </x:c>
       <x:c r="I14" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>ADM-M-013; ADM-M-019</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
         <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K14" s="10" t="str"/>
       <x:c r="L14" s="10" t="str">
-        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
+        <x:v>The migration parsed and applied to a fresh disposable local PostgreSQL schema. Atomic replay and rollback plus direct actor/tamper/expiry denials passed. This is isolated local evidence, not dedicated Supabase staging or a complete Org A/Org B matrix.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
+        <x:v>EVD-SEC104-SITEMAP-LOCAL</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20766,31 +20764,31 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E15" s="12" t="n">
-        <x:v>46262.33998842593</x:v>
+        <x:v>46262.3490625</x:v>
       </x:c>
       <x:c r="F15" s="10" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="G15" s="10" t="str">
-        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>c50c597d0c24e745d3601b085a7a1daf1d32ad67</x:v>
       </x:c>
       <x:c r="H15" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
+        <x:v>Node 20 route registry, SEC-104 focused Vitest, complete Admin Vitest, touched ESLint, and scoped TypeScript commands recorded in TASK_LOG.md</x:v>
       </x:c>
       <x:c r="I15" s="10" t="str">
-        <x:v>AOA-012</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-013; ADM-WF-017</x:v>
       </x:c>
       <x:c r="K15" s="10" t="str"/>
       <x:c r="L15" s="10" t="str">
-        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
+        <x:v>Local verification passed: exact 288 routes at 114/114 legacy; 9 focused tests; 228 active Admin files and 3,206 active Admin tests; touched lint and scoped TypeScript. One live-security file and two environment-dependent tests remain skipped, and no staging evidence is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-WAVE0-ADMIN-TESTS-LOCAL</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20802,7 +20800,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E16" s="12" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.33998842593</x:v>
       </x:c>
       <x:c r="F16" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20811,25 +20809,25 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H16" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node node_modules/vitest/vitest.mjs run __tests__/admin</x:v>
       </x:c>
       <x:c r="I16" s="10" t="str">
-        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
+        <x:v>AOA-012</x:v>
       </x:c>
       <x:c r="J16" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K16" s="10" t="str"/>
       <x:c r="L16" s="10" t="str">
-        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
+        <x:v>Local pinned-toolchain run: 227 test files passed, 1 file skipped; 3,203 tests passed and 2 tests skipped. The skipped live/environment security cases remain unverified and prevent this receipt from satisfying LG-03.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
+        <x:v>EVD-WAVE0-AUDIT-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>commit</x:v>
+        <x:v>test_run</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
         <x:v>pass</x:v>
@@ -20838,7 +20836,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E17" s="12" t="n">
-        <x:v>46262.33961805556</x:v>
+        <x:v>46262.339895833335</x:v>
       </x:c>
       <x:c r="F17" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20847,25 +20845,25 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H17" s="10" t="str">
-        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --import tsx scripts/audit/admin-workflow-registry.ts --check --require-workbook</x:v>
       </x:c>
       <x:c r="I17" s="10" t="str">
-        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
+        <x:v>AOA-001; AOA-004; AOA-005; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K17" s="10" t="str"/>
       <x:c r="L17" s="10" t="str">
-        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
+        <x:v>Local registry validation passed for 79 findings, 362 specification tasks, 20 workflows, 18 launch gates, the generated views, and the workbook manifest. Local evidence is intentionally not attached to a CI launch gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
+        <x:v>EVD-WAVE0-CONTROLS-COMMIT</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>test_run</x:v>
+        <x:v>commit</x:v>
       </x:c>
       <x:c r="C18" s="10" t="str">
         <x:v>pass</x:v>
@@ -20874,7 +20872,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="E18" s="12" t="n">
-        <x:v>46262.339895833335</x:v>
+        <x:v>46262.33961805556</x:v>
       </x:c>
       <x:c r="F18" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20883,22 +20881,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H18" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
+        <x:v>git:codex/admin-workflow-completion@8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="I18" s="10" t="str">
-        <x:v>AOA-013; AOA-015</x:v>
+        <x:v>ADM-M-013; AOA-001; AOA-002; AOA-004; AOA-005; AOA-006; AOA-008; AOA-009; AOA-010; AOA-011; AOA-014; AOA-015</x:v>
       </x:c>
       <x:c r="J18" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K18" s="10" t="str"/>
       <x:c r="L18" s="10" t="str">
-        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
+        <x:v>Immutable implementation checkpoint for the Wave 0 registry, route contracts, service-role classification, migration validation, and baseline test repairs. This is implementation evidence, not CI, staging, or independent-verification evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="A19" s="10" t="str">
-        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
+        <x:v>EVD-WAVE0-MIGRATIONS-LOCAL</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20919,22 +20917,22 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H19" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-migration-validation.mjs</x:v>
       </x:c>
       <x:c r="I19" s="10" t="str">
-        <x:v>ADM-M-013</x:v>
+        <x:v>AOA-013; AOA-015</x:v>
       </x:c>
       <x:c r="J19" s="10" t="str">
         <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K19" s="10" t="str"/>
       <x:c r="L19" s="10" t="str">
-        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
+        <x:v>Repository migration scanner passed against immutable historical checksums and declared planned/isolated manifests. No migration was applied to a fresh or staging Supabase project, so parity and live provenance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="46" customHeight="1">
       <x:c r="A20" s="10" t="str">
-        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
+        <x:v>EVD-WAVE0-ROUTE-REGISTRY-LOCAL</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
         <x:v>test_run</x:v>
@@ -20955,34 +20953,34 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H20" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-admin-route-registry.mjs</x:v>
       </x:c>
       <x:c r="I20" s="10" t="str">
         <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J20" s="10" t="str">
-        <x:v>ADM-WF-017; ADM-WF-019</x:v>
+        <x:v>ADM-WF-017</x:v>
       </x:c>
       <x:c r="K20" s="10" t="str"/>
       <x:c r="L20" s="10" t="str">
-        <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
+        <x:v>Local route inventory passed with 288 Admin API route files and an exact 117/117 legacy ceiling. Runtime capability, tenant-denial, idempotency, and audit-event evidence remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="46" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+        <x:v>EVD-WAVE0-SERVICE-ROLE-LOCAL</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
         <x:v>test_run</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
-        <x:v>fail</x:v>
+        <x:v>pass</x:v>
       </x:c>
       <x:c r="D21" s="10" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="E21" s="12" t="n">
-        <x:v>46262.33513888889</x:v>
+        <x:v>46262.339895833335</x:v>
       </x:c>
       <x:c r="F21" s="10" t="str">
         <x:v>Codex</x:v>
@@ -20991,27 +20989,63 @@
         <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
       </x:c>
       <x:c r="H21" s="10" t="str">
-        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node scripts/ci/check-service-role-allowlist.mjs</x:v>
       </x:c>
       <x:c r="I21" s="10" t="str">
-        <x:v>ADM-M-001; AOA-003</x:v>
+        <x:v>ADM-M-013</x:v>
       </x:c>
       <x:c r="J21" s="10" t="str">
-        <x:v>ADM-WF-017</x:v>
+        <x:v>ADM-WF-017; ADM-WF-019</x:v>
       </x:c>
       <x:c r="K21" s="10" t="str"/>
       <x:c r="L21" s="10" t="str">
+        <x:v>Local classification gate passed for 168 production files: 144 historical entries, 23 reviewed remediation-debt entries, and 1 low-level factory. This does not close the underlying migration debt or prove live actor binding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="46" customHeight="1">
+      <x:c r="A22" s="10" t="str">
+        <x:v>EVD-WAVE0-TYPECHECK-LOCAL-FAIL</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>test_run</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>fail</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="n">
+        <x:v>46262.33513888889</x:v>
+      </x:c>
+      <x:c r="F22" s="10" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="G22" s="10" t="str">
+        <x:v>8c40df23a4995088cf88ea69bf809035f0c3de28</x:v>
+      </x:c>
+      <x:c r="H22" s="10" t="str">
+        <x:v>/Users/kyledaley/.nvm/versions/node/v20.20.2/bin/node --max-old-space-size=8192 node_modules/typescript/bin/tsc --noEmit --pretty false --incremental false --diagnostics</x:v>
+      </x:c>
+      <x:c r="I22" s="10" t="str">
+        <x:v>ADM-M-001; AOA-003</x:v>
+      </x:c>
+      <x:c r="J22" s="10" t="str">
+        <x:v>ADM-WF-017</x:v>
+      </x:c>
+      <x:c r="K22" s="10" t="str"/>
+      <x:c r="L22" s="10" t="str">
         <x:v>Pinned Node 20 full-repository typecheck exited 2 after 2,652.36 seconds. It checked 7,456 files, used about 6.3 GB, and reported type/schema drift across Admin and non-Admin code; the captured command output contained 3,005 lines. LG-01 remains not verified and the production build was not attempted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C21">
+  <x:conditionalFormatting sqref="C2:C22">
     <x:cfRule type="containsText" dxfId="49" priority="1" operator="containsText" text="pass"/>
     <x:cfRule type="containsText" dxfId="50" priority="2" operator="containsText" text="fail"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc662ace99b574c48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2320ff852764aea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21265,7 +21299,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re197fa39fc1e46ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34d98470abb34909"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>